<commit_message>
feat(goal-engine): complete T006 goal engine integration
</commit_message>
<xml_diff>
--- a/workbook/FinanceOS_v1.0.xlsx
+++ b/workbook/FinanceOS_v1.0.xlsx
@@ -1710,7 +1710,9 @@
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Goal Category"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Goal Account"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="Target Amount"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="Current Saved Amount"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="Current Saved Amount">
+      <calculatedColumnFormula>IF(tblGoals[[#This Row],[Goal ID]]="","",IFERROR(SUMPRODUCT((tblTransactions[Transaction Type]="Expense")*(tblTransactions[Destination Type]="Goal")*((tblTransactions[Transaction Status]="Completed")+(tblTransactions[Transaction Status]="Reconciled"))*(IFERROR(INDEX(tblGoals[Goal ID],MATCH(tblTransactions[Destination Name],tblGoals[Goal ID],0)),IFERROR(INDEX(tblGoals[Goal ID],MATCH(tblTransactions[Destination Name],tblGoals[Goal Name],0)),""))=tblGoals[[#This Row],[Goal ID]])*(tblTransactions[Amount])),0))</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Remaining Amount">
       <calculatedColumnFormula>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</calculatedColumnFormula>
     </tableColumn>
@@ -33673,7 +33675,9 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="1"/>
+      <c r="F2" s="1">
+        <f t="shared" ref="F2:F200" si="0">IF(tblGoals[[#This Row],[Goal ID]]="","",IFERROR(SUMPRODUCT((tblTransactions[Transaction Type]="Expense")*(tblTransactions[Destination Type]="Goal")*((tblTransactions[Transaction Status]="Completed")+(tblTransactions[Transaction Status]="Reconciled"))*(IFERROR(INDEX(tblGoals[Goal ID],MATCH(tblTransactions[Destination Name],tblGoals[Goal ID],0)),IFERROR(INDEX(tblGoals[Goal ID],MATCH(tblTransactions[Destination Name],tblGoals[Goal Name],0)),""))=tblGoals[[#This Row],[Goal ID]])*(tblTransactions[Amount])),0))</f>
+      </c>
       <c r="G2" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33690,7 +33694,9 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="1"/>
+      <c r="F3" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G3" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33707,7 +33713,9 @@
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="1"/>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G4" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33724,7 +33732,9 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="1"/>
+      <c r="F5" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G5" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33741,7 +33751,9 @@
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="1"/>
+      <c r="F6" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G6" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33758,7 +33770,9 @@
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
-      <c r="F7" s="1"/>
+      <c r="F7" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G7" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33775,7 +33789,9 @@
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="1"/>
+      <c r="F8" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G8" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33792,7 +33808,9 @@
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="1"/>
+      <c r="F9" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G9" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33809,7 +33827,9 @@
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="F10" s="1"/>
+      <c r="F10" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G10" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33826,7 +33846,9 @@
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="F11" s="1"/>
+      <c r="F11" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G11" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33843,7 +33865,9 @@
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="1"/>
+      <c r="F12" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G12" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33860,7 +33884,9 @@
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="1"/>
+      <c r="F13" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G13" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33877,7 +33903,9 @@
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
-      <c r="F14" s="1"/>
+      <c r="F14" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G14" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33894,7 +33922,9 @@
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
-      <c r="F15" s="1"/>
+      <c r="F15" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G15" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33911,7 +33941,9 @@
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
-      <c r="F16" s="1"/>
+      <c r="F16" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G16" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33928,7 +33960,9 @@
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
-      <c r="F17" s="1"/>
+      <c r="F17" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G17" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33945,7 +33979,9 @@
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
-      <c r="F18" s="1"/>
+      <c r="F18" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G18" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33962,7 +33998,9 @@
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="1"/>
+      <c r="F19" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G19" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33979,7 +34017,9 @@
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
-      <c r="F20" s="1"/>
+      <c r="F20" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G20" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -33996,7 +34036,9 @@
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
-      <c r="F21" s="1"/>
+      <c r="F21" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G21" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34013,7 +34055,9 @@
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
-      <c r="F22" s="1"/>
+      <c r="F22" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G22" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34030,7 +34074,9 @@
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
-      <c r="F23" s="1"/>
+      <c r="F23" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G23" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34047,7 +34093,9 @@
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
-      <c r="F24" s="1"/>
+      <c r="F24" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G24" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34064,7 +34112,9 @@
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
-      <c r="F25" s="1"/>
+      <c r="F25" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G25" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34081,7 +34131,9 @@
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
-      <c r="F26" s="1"/>
+      <c r="F26" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G26" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34098,7 +34150,9 @@
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
-      <c r="F27" s="1"/>
+      <c r="F27" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G27" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34115,7 +34169,9 @@
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
-      <c r="F28" s="1"/>
+      <c r="F28" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G28" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34132,7 +34188,9 @@
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
-      <c r="F29" s="1"/>
+      <c r="F29" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G29" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34149,7 +34207,9 @@
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
-      <c r="F30" s="1"/>
+      <c r="F30" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G30" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34166,7 +34226,9 @@
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
-      <c r="F31" s="1"/>
+      <c r="F31" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G31" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34183,7 +34245,9 @@
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
-      <c r="F32" s="1"/>
+      <c r="F32" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G32" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34200,7 +34264,9 @@
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
-      <c r="F33" s="1"/>
+      <c r="F33" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G33" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34217,7 +34283,9 @@
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
-      <c r="F34" s="1"/>
+      <c r="F34" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G34" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34234,7 +34302,9 @@
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
-      <c r="F35" s="1"/>
+      <c r="F35" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G35" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34251,7 +34321,9 @@
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
-      <c r="F36" s="1"/>
+      <c r="F36" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G36" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34268,7 +34340,9 @@
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
-      <c r="F37" s="1"/>
+      <c r="F37" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G37" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34285,7 +34359,9 @@
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
-      <c r="F38" s="1"/>
+      <c r="F38" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G38" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34302,7 +34378,9 @@
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
-      <c r="F39" s="1"/>
+      <c r="F39" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G39" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34319,7 +34397,9 @@
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
-      <c r="F40" s="1"/>
+      <c r="F40" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G40" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34336,7 +34416,9 @@
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
-      <c r="F41" s="1"/>
+      <c r="F41" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G41" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34353,7 +34435,9 @@
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
-      <c r="F42" s="1"/>
+      <c r="F42" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G42" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34370,7 +34454,9 @@
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
-      <c r="F43" s="1"/>
+      <c r="F43" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G43" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34387,7 +34473,9 @@
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
-      <c r="F44" s="1"/>
+      <c r="F44" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G44" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34404,7 +34492,9 @@
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
-      <c r="F45" s="1"/>
+      <c r="F45" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G45" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34421,7 +34511,9 @@
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
-      <c r="F46" s="1"/>
+      <c r="F46" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G46" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34438,7 +34530,9 @@
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
-      <c r="F47" s="1"/>
+      <c r="F47" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G47" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34455,7 +34549,9 @@
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
-      <c r="F48" s="1"/>
+      <c r="F48" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G48" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34472,7 +34568,9 @@
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
-      <c r="F49" s="1"/>
+      <c r="F49" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G49" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34489,7 +34587,9 @@
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
-      <c r="F50" s="1"/>
+      <c r="F50" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G50" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34506,7 +34606,9 @@
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
-      <c r="F51" s="1"/>
+      <c r="F51" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G51" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34523,7 +34625,9 @@
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
-      <c r="F52" s="1"/>
+      <c r="F52" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G52" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34540,7 +34644,9 @@
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
-      <c r="F53" s="1"/>
+      <c r="F53" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G53" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34557,7 +34663,9 @@
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
-      <c r="F54" s="1"/>
+      <c r="F54" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G54" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34574,7 +34682,9 @@
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
-      <c r="F55" s="1"/>
+      <c r="F55" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G55" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34591,7 +34701,9 @@
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
-      <c r="F56" s="1"/>
+      <c r="F56" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G56" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34608,7 +34720,9 @@
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
-      <c r="F57" s="1"/>
+      <c r="F57" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G57" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34625,7 +34739,9 @@
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
-      <c r="F58" s="1"/>
+      <c r="F58" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G58" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34642,7 +34758,9 @@
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
-      <c r="F59" s="1"/>
+      <c r="F59" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G59" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34659,7 +34777,9 @@
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
-      <c r="F60" s="1"/>
+      <c r="F60" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G60" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34676,7 +34796,9 @@
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="2"/>
-      <c r="F61" s="1"/>
+      <c r="F61" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G61" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34693,7 +34815,9 @@
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
       <c r="E62" s="2"/>
-      <c r="F62" s="1"/>
+      <c r="F62" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G62" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34710,7 +34834,9 @@
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
-      <c r="F63" s="1"/>
+      <c r="F63" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G63" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34727,7 +34853,9 @@
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
-      <c r="F64" s="1"/>
+      <c r="F64" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G64" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34744,7 +34872,9 @@
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
-      <c r="F65" s="1"/>
+      <c r="F65" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G65" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34761,7 +34891,9 @@
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
-      <c r="F66" s="1"/>
+      <c r="F66" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G66" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34778,7 +34910,9 @@
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
-      <c r="F67" s="1"/>
+      <c r="F67" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G67" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34795,7 +34929,9 @@
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
       <c r="E68" s="2"/>
-      <c r="F68" s="1"/>
+      <c r="F68" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G68" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34812,7 +34948,9 @@
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
       <c r="E69" s="2"/>
-      <c r="F69" s="1"/>
+      <c r="F69" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G69" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34829,7 +34967,9 @@
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
       <c r="E70" s="2"/>
-      <c r="F70" s="1"/>
+      <c r="F70" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G70" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34846,7 +34986,9 @@
       <c r="C71" s="2"/>
       <c r="D71" s="2"/>
       <c r="E71" s="2"/>
-      <c r="F71" s="1"/>
+      <c r="F71" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G71" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34863,7 +35005,9 @@
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
       <c r="E72" s="2"/>
-      <c r="F72" s="1"/>
+      <c r="F72" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G72" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34880,7 +35024,9 @@
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
       <c r="E73" s="2"/>
-      <c r="F73" s="1"/>
+      <c r="F73" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G73" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34897,7 +35043,9 @@
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
       <c r="E74" s="2"/>
-      <c r="F74" s="1"/>
+      <c r="F74" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G74" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34914,7 +35062,9 @@
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
       <c r="E75" s="2"/>
-      <c r="F75" s="1"/>
+      <c r="F75" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G75" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34931,7 +35081,9 @@
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
       <c r="E76" s="2"/>
-      <c r="F76" s="1"/>
+      <c r="F76" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G76" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34948,7 +35100,9 @@
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
       <c r="E77" s="2"/>
-      <c r="F77" s="1"/>
+      <c r="F77" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G77" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34965,7 +35119,9 @@
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2"/>
-      <c r="F78" s="1"/>
+      <c r="F78" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G78" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34982,7 +35138,9 @@
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2"/>
-      <c r="F79" s="1"/>
+      <c r="F79" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G79" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -34999,7 +35157,9 @@
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2"/>
-      <c r="F80" s="1"/>
+      <c r="F80" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G80" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35016,7 +35176,9 @@
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2"/>
-      <c r="F81" s="1"/>
+      <c r="F81" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G81" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35033,7 +35195,9 @@
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
       <c r="E82" s="2"/>
-      <c r="F82" s="1"/>
+      <c r="F82" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G82" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35050,7 +35214,9 @@
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2"/>
-      <c r="F83" s="1"/>
+      <c r="F83" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G83" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35067,7 +35233,9 @@
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
       <c r="E84" s="2"/>
-      <c r="F84" s="1"/>
+      <c r="F84" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G84" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35084,7 +35252,9 @@
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
       <c r="E85" s="2"/>
-      <c r="F85" s="1"/>
+      <c r="F85" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G85" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35101,7 +35271,9 @@
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
       <c r="E86" s="2"/>
-      <c r="F86" s="1"/>
+      <c r="F86" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G86" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35118,7 +35290,9 @@
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
-      <c r="F87" s="1"/>
+      <c r="F87" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G87" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35135,7 +35309,9 @@
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
       <c r="E88" s="2"/>
-      <c r="F88" s="1"/>
+      <c r="F88" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G88" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35152,7 +35328,9 @@
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
       <c r="E89" s="2"/>
-      <c r="F89" s="1"/>
+      <c r="F89" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G89" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35169,7 +35347,9 @@
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
       <c r="E90" s="2"/>
-      <c r="F90" s="1"/>
+      <c r="F90" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G90" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35186,7 +35366,9 @@
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
       <c r="E91" s="2"/>
-      <c r="F91" s="1"/>
+      <c r="F91" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G91" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35203,7 +35385,9 @@
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
       <c r="E92" s="2"/>
-      <c r="F92" s="1"/>
+      <c r="F92" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G92" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35220,7 +35404,9 @@
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
       <c r="E93" s="2"/>
-      <c r="F93" s="1"/>
+      <c r="F93" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G93" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35237,7 +35423,9 @@
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
       <c r="E94" s="2"/>
-      <c r="F94" s="1"/>
+      <c r="F94" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G94" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35254,7 +35442,9 @@
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
       <c r="E95" s="2"/>
-      <c r="F95" s="1"/>
+      <c r="F95" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G95" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35271,7 +35461,9 @@
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
       <c r="E96" s="2"/>
-      <c r="F96" s="1"/>
+      <c r="F96" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G96" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35288,7 +35480,9 @@
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
-      <c r="F97" s="1"/>
+      <c r="F97" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G97" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35305,7 +35499,9 @@
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
       <c r="E98" s="2"/>
-      <c r="F98" s="1"/>
+      <c r="F98" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G98" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35322,7 +35518,9 @@
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
       <c r="E99" s="2"/>
-      <c r="F99" s="1"/>
+      <c r="F99" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G99" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35339,7 +35537,9 @@
       <c r="C100" s="2"/>
       <c r="D100" s="2"/>
       <c r="E100" s="2"/>
-      <c r="F100" s="1"/>
+      <c r="F100" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G100" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35356,7 +35556,9 @@
       <c r="C101" s="2"/>
       <c r="D101" s="2"/>
       <c r="E101" s="2"/>
-      <c r="F101" s="1"/>
+      <c r="F101" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G101" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35373,7 +35575,9 @@
       <c r="C102" s="2"/>
       <c r="D102" s="2"/>
       <c r="E102" s="2"/>
-      <c r="F102" s="1"/>
+      <c r="F102" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G102" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35390,7 +35594,9 @@
       <c r="C103" s="2"/>
       <c r="D103" s="2"/>
       <c r="E103" s="2"/>
-      <c r="F103" s="1"/>
+      <c r="F103" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G103" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35407,7 +35613,9 @@
       <c r="C104" s="2"/>
       <c r="D104" s="2"/>
       <c r="E104" s="2"/>
-      <c r="F104" s="1"/>
+      <c r="F104" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G104" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35424,7 +35632,9 @@
       <c r="C105" s="2"/>
       <c r="D105" s="2"/>
       <c r="E105" s="2"/>
-      <c r="F105" s="1"/>
+      <c r="F105" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G105" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35441,7 +35651,9 @@
       <c r="C106" s="2"/>
       <c r="D106" s="2"/>
       <c r="E106" s="2"/>
-      <c r="F106" s="1"/>
+      <c r="F106" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G106" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35458,7 +35670,9 @@
       <c r="C107" s="2"/>
       <c r="D107" s="2"/>
       <c r="E107" s="2"/>
-      <c r="F107" s="1"/>
+      <c r="F107" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G107" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35475,7 +35689,9 @@
       <c r="C108" s="2"/>
       <c r="D108" s="2"/>
       <c r="E108" s="2"/>
-      <c r="F108" s="1"/>
+      <c r="F108" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G108" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35492,7 +35708,9 @@
       <c r="C109" s="2"/>
       <c r="D109" s="2"/>
       <c r="E109" s="2"/>
-      <c r="F109" s="1"/>
+      <c r="F109" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G109" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35509,7 +35727,9 @@
       <c r="C110" s="2"/>
       <c r="D110" s="2"/>
       <c r="E110" s="2"/>
-      <c r="F110" s="1"/>
+      <c r="F110" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G110" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35526,7 +35746,9 @@
       <c r="C111" s="2"/>
       <c r="D111" s="2"/>
       <c r="E111" s="2"/>
-      <c r="F111" s="1"/>
+      <c r="F111" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G111" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35543,7 +35765,9 @@
       <c r="C112" s="2"/>
       <c r="D112" s="2"/>
       <c r="E112" s="2"/>
-      <c r="F112" s="1"/>
+      <c r="F112" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G112" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35560,7 +35784,9 @@
       <c r="C113" s="2"/>
       <c r="D113" s="2"/>
       <c r="E113" s="2"/>
-      <c r="F113" s="1"/>
+      <c r="F113" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G113" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35577,7 +35803,9 @@
       <c r="C114" s="2"/>
       <c r="D114" s="2"/>
       <c r="E114" s="2"/>
-      <c r="F114" s="1"/>
+      <c r="F114" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G114" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35594,7 +35822,9 @@
       <c r="C115" s="2"/>
       <c r="D115" s="2"/>
       <c r="E115" s="2"/>
-      <c r="F115" s="1"/>
+      <c r="F115" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G115" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35611,7 +35841,9 @@
       <c r="C116" s="2"/>
       <c r="D116" s="2"/>
       <c r="E116" s="2"/>
-      <c r="F116" s="1"/>
+      <c r="F116" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G116" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35628,7 +35860,9 @@
       <c r="C117" s="2"/>
       <c r="D117" s="2"/>
       <c r="E117" s="2"/>
-      <c r="F117" s="1"/>
+      <c r="F117" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G117" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35645,7 +35879,9 @@
       <c r="C118" s="2"/>
       <c r="D118" s="2"/>
       <c r="E118" s="2"/>
-      <c r="F118" s="1"/>
+      <c r="F118" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G118" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35662,7 +35898,9 @@
       <c r="C119" s="2"/>
       <c r="D119" s="2"/>
       <c r="E119" s="2"/>
-      <c r="F119" s="1"/>
+      <c r="F119" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G119" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35679,7 +35917,9 @@
       <c r="C120" s="2"/>
       <c r="D120" s="2"/>
       <c r="E120" s="2"/>
-      <c r="F120" s="1"/>
+      <c r="F120" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G120" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35696,7 +35936,9 @@
       <c r="C121" s="2"/>
       <c r="D121" s="2"/>
       <c r="E121" s="2"/>
-      <c r="F121" s="1"/>
+      <c r="F121" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G121" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35713,7 +35955,9 @@
       <c r="C122" s="2"/>
       <c r="D122" s="2"/>
       <c r="E122" s="2"/>
-      <c r="F122" s="1"/>
+      <c r="F122" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G122" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35730,7 +35974,9 @@
       <c r="C123" s="2"/>
       <c r="D123" s="2"/>
       <c r="E123" s="2"/>
-      <c r="F123" s="1"/>
+      <c r="F123" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G123" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35747,7 +35993,9 @@
       <c r="C124" s="2"/>
       <c r="D124" s="2"/>
       <c r="E124" s="2"/>
-      <c r="F124" s="1"/>
+      <c r="F124" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G124" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35764,7 +36012,9 @@
       <c r="C125" s="2"/>
       <c r="D125" s="2"/>
       <c r="E125" s="2"/>
-      <c r="F125" s="1"/>
+      <c r="F125" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G125" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35781,7 +36031,9 @@
       <c r="C126" s="2"/>
       <c r="D126" s="2"/>
       <c r="E126" s="2"/>
-      <c r="F126" s="1"/>
+      <c r="F126" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G126" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35798,7 +36050,9 @@
       <c r="C127" s="2"/>
       <c r="D127" s="2"/>
       <c r="E127" s="2"/>
-      <c r="F127" s="1"/>
+      <c r="F127" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G127" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35815,7 +36069,9 @@
       <c r="C128" s="2"/>
       <c r="D128" s="2"/>
       <c r="E128" s="2"/>
-      <c r="F128" s="1"/>
+      <c r="F128" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G128" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35832,7 +36088,9 @@
       <c r="C129" s="2"/>
       <c r="D129" s="2"/>
       <c r="E129" s="2"/>
-      <c r="F129" s="1"/>
+      <c r="F129" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G129" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35849,7 +36107,9 @@
       <c r="C130" s="2"/>
       <c r="D130" s="2"/>
       <c r="E130" s="2"/>
-      <c r="F130" s="1"/>
+      <c r="F130" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G130" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35866,7 +36126,9 @@
       <c r="C131" s="2"/>
       <c r="D131" s="2"/>
       <c r="E131" s="2"/>
-      <c r="F131" s="1"/>
+      <c r="F131" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G131" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35883,7 +36145,9 @@
       <c r="C132" s="2"/>
       <c r="D132" s="2"/>
       <c r="E132" s="2"/>
-      <c r="F132" s="1"/>
+      <c r="F132" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G132" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35900,7 +36164,9 @@
       <c r="C133" s="2"/>
       <c r="D133" s="2"/>
       <c r="E133" s="2"/>
-      <c r="F133" s="1"/>
+      <c r="F133" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G133" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35917,7 +36183,9 @@
       <c r="C134" s="2"/>
       <c r="D134" s="2"/>
       <c r="E134" s="2"/>
-      <c r="F134" s="1"/>
+      <c r="F134" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G134" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35934,7 +36202,9 @@
       <c r="C135" s="2"/>
       <c r="D135" s="2"/>
       <c r="E135" s="2"/>
-      <c r="F135" s="1"/>
+      <c r="F135" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G135" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35951,7 +36221,9 @@
       <c r="C136" s="2"/>
       <c r="D136" s="2"/>
       <c r="E136" s="2"/>
-      <c r="F136" s="1"/>
+      <c r="F136" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G136" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35968,7 +36240,9 @@
       <c r="C137" s="2"/>
       <c r="D137" s="2"/>
       <c r="E137" s="2"/>
-      <c r="F137" s="1"/>
+      <c r="F137" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G137" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -35985,7 +36259,9 @@
       <c r="C138" s="2"/>
       <c r="D138" s="2"/>
       <c r="E138" s="2"/>
-      <c r="F138" s="1"/>
+      <c r="F138" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G138" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36002,7 +36278,9 @@
       <c r="C139" s="2"/>
       <c r="D139" s="2"/>
       <c r="E139" s="2"/>
-      <c r="F139" s="1"/>
+      <c r="F139" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G139" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36019,7 +36297,9 @@
       <c r="C140" s="2"/>
       <c r="D140" s="2"/>
       <c r="E140" s="2"/>
-      <c r="F140" s="1"/>
+      <c r="F140" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G140" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36036,7 +36316,9 @@
       <c r="C141" s="2"/>
       <c r="D141" s="2"/>
       <c r="E141" s="2"/>
-      <c r="F141" s="1"/>
+      <c r="F141" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G141" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36053,7 +36335,9 @@
       <c r="C142" s="2"/>
       <c r="D142" s="2"/>
       <c r="E142" s="2"/>
-      <c r="F142" s="1"/>
+      <c r="F142" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G142" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36070,7 +36354,9 @@
       <c r="C143" s="2"/>
       <c r="D143" s="2"/>
       <c r="E143" s="2"/>
-      <c r="F143" s="1"/>
+      <c r="F143" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G143" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36087,7 +36373,9 @@
       <c r="C144" s="2"/>
       <c r="D144" s="2"/>
       <c r="E144" s="2"/>
-      <c r="F144" s="1"/>
+      <c r="F144" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G144" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36104,7 +36392,9 @@
       <c r="C145" s="2"/>
       <c r="D145" s="2"/>
       <c r="E145" s="2"/>
-      <c r="F145" s="1"/>
+      <c r="F145" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G145" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36121,7 +36411,9 @@
       <c r="C146" s="2"/>
       <c r="D146" s="2"/>
       <c r="E146" s="2"/>
-      <c r="F146" s="1"/>
+      <c r="F146" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G146" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36138,7 +36430,9 @@
       <c r="C147" s="2"/>
       <c r="D147" s="2"/>
       <c r="E147" s="2"/>
-      <c r="F147" s="1"/>
+      <c r="F147" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G147" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36155,7 +36449,9 @@
       <c r="C148" s="2"/>
       <c r="D148" s="2"/>
       <c r="E148" s="2"/>
-      <c r="F148" s="1"/>
+      <c r="F148" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G148" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36172,7 +36468,9 @@
       <c r="C149" s="2"/>
       <c r="D149" s="2"/>
       <c r="E149" s="2"/>
-      <c r="F149" s="1"/>
+      <c r="F149" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G149" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36189,7 +36487,9 @@
       <c r="C150" s="2"/>
       <c r="D150" s="2"/>
       <c r="E150" s="2"/>
-      <c r="F150" s="1"/>
+      <c r="F150" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G150" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36206,7 +36506,9 @@
       <c r="C151" s="2"/>
       <c r="D151" s="2"/>
       <c r="E151" s="2"/>
-      <c r="F151" s="1"/>
+      <c r="F151" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G151" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36223,7 +36525,9 @@
       <c r="C152" s="2"/>
       <c r="D152" s="2"/>
       <c r="E152" s="2"/>
-      <c r="F152" s="1"/>
+      <c r="F152" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G152" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36240,7 +36544,9 @@
       <c r="C153" s="2"/>
       <c r="D153" s="2"/>
       <c r="E153" s="2"/>
-      <c r="F153" s="1"/>
+      <c r="F153" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G153" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36257,7 +36563,9 @@
       <c r="C154" s="2"/>
       <c r="D154" s="2"/>
       <c r="E154" s="2"/>
-      <c r="F154" s="1"/>
+      <c r="F154" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G154" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36274,7 +36582,9 @@
       <c r="C155" s="2"/>
       <c r="D155" s="2"/>
       <c r="E155" s="2"/>
-      <c r="F155" s="1"/>
+      <c r="F155" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G155" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36291,7 +36601,9 @@
       <c r="C156" s="2"/>
       <c r="D156" s="2"/>
       <c r="E156" s="2"/>
-      <c r="F156" s="1"/>
+      <c r="F156" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G156" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36308,7 +36620,9 @@
       <c r="C157" s="2"/>
       <c r="D157" s="2"/>
       <c r="E157" s="2"/>
-      <c r="F157" s="1"/>
+      <c r="F157" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G157" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36325,7 +36639,9 @@
       <c r="C158" s="2"/>
       <c r="D158" s="2"/>
       <c r="E158" s="2"/>
-      <c r="F158" s="1"/>
+      <c r="F158" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G158" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36342,7 +36658,9 @@
       <c r="C159" s="2"/>
       <c r="D159" s="2"/>
       <c r="E159" s="2"/>
-      <c r="F159" s="1"/>
+      <c r="F159" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G159" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36359,7 +36677,9 @@
       <c r="C160" s="2"/>
       <c r="D160" s="2"/>
       <c r="E160" s="2"/>
-      <c r="F160" s="1"/>
+      <c r="F160" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G160" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36376,7 +36696,9 @@
       <c r="C161" s="2"/>
       <c r="D161" s="2"/>
       <c r="E161" s="2"/>
-      <c r="F161" s="1"/>
+      <c r="F161" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G161" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36393,7 +36715,9 @@
       <c r="C162" s="2"/>
       <c r="D162" s="2"/>
       <c r="E162" s="2"/>
-      <c r="F162" s="1"/>
+      <c r="F162" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G162" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36410,7 +36734,9 @@
       <c r="C163" s="2"/>
       <c r="D163" s="2"/>
       <c r="E163" s="2"/>
-      <c r="F163" s="1"/>
+      <c r="F163" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G163" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36427,7 +36753,9 @@
       <c r="C164" s="2"/>
       <c r="D164" s="2"/>
       <c r="E164" s="2"/>
-      <c r="F164" s="1"/>
+      <c r="F164" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G164" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36444,7 +36772,9 @@
       <c r="C165" s="2"/>
       <c r="D165" s="2"/>
       <c r="E165" s="2"/>
-      <c r="F165" s="1"/>
+      <c r="F165" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G165" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36461,7 +36791,9 @@
       <c r="C166" s="2"/>
       <c r="D166" s="2"/>
       <c r="E166" s="2"/>
-      <c r="F166" s="1"/>
+      <c r="F166" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G166" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36478,7 +36810,9 @@
       <c r="C167" s="2"/>
       <c r="D167" s="2"/>
       <c r="E167" s="2"/>
-      <c r="F167" s="1"/>
+      <c r="F167" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G167" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36495,7 +36829,9 @@
       <c r="C168" s="2"/>
       <c r="D168" s="2"/>
       <c r="E168" s="2"/>
-      <c r="F168" s="1"/>
+      <c r="F168" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G168" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36512,7 +36848,9 @@
       <c r="C169" s="2"/>
       <c r="D169" s="2"/>
       <c r="E169" s="2"/>
-      <c r="F169" s="1"/>
+      <c r="F169" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G169" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36529,7 +36867,9 @@
       <c r="C170" s="2"/>
       <c r="D170" s="2"/>
       <c r="E170" s="2"/>
-      <c r="F170" s="1"/>
+      <c r="F170" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G170" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36546,7 +36886,9 @@
       <c r="C171" s="2"/>
       <c r="D171" s="2"/>
       <c r="E171" s="2"/>
-      <c r="F171" s="1"/>
+      <c r="F171" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G171" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36563,7 +36905,9 @@
       <c r="C172" s="2"/>
       <c r="D172" s="2"/>
       <c r="E172" s="2"/>
-      <c r="F172" s="1"/>
+      <c r="F172" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G172" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36580,7 +36924,9 @@
       <c r="C173" s="2"/>
       <c r="D173" s="2"/>
       <c r="E173" s="2"/>
-      <c r="F173" s="1"/>
+      <c r="F173" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G173" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36597,7 +36943,9 @@
       <c r="C174" s="2"/>
       <c r="D174" s="2"/>
       <c r="E174" s="2"/>
-      <c r="F174" s="1"/>
+      <c r="F174" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G174" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36614,7 +36962,9 @@
       <c r="C175" s="2"/>
       <c r="D175" s="2"/>
       <c r="E175" s="2"/>
-      <c r="F175" s="1"/>
+      <c r="F175" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G175" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36631,7 +36981,9 @@
       <c r="C176" s="2"/>
       <c r="D176" s="2"/>
       <c r="E176" s="2"/>
-      <c r="F176" s="1"/>
+      <c r="F176" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G176" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36648,7 +37000,9 @@
       <c r="C177" s="2"/>
       <c r="D177" s="2"/>
       <c r="E177" s="2"/>
-      <c r="F177" s="1"/>
+      <c r="F177" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G177" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36665,7 +37019,9 @@
       <c r="C178" s="2"/>
       <c r="D178" s="2"/>
       <c r="E178" s="2"/>
-      <c r="F178" s="1"/>
+      <c r="F178" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G178" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36682,7 +37038,9 @@
       <c r="C179" s="2"/>
       <c r="D179" s="2"/>
       <c r="E179" s="2"/>
-      <c r="F179" s="1"/>
+      <c r="F179" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G179" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36699,7 +37057,9 @@
       <c r="C180" s="2"/>
       <c r="D180" s="2"/>
       <c r="E180" s="2"/>
-      <c r="F180" s="1"/>
+      <c r="F180" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G180" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36716,7 +37076,9 @@
       <c r="C181" s="2"/>
       <c r="D181" s="2"/>
       <c r="E181" s="2"/>
-      <c r="F181" s="1"/>
+      <c r="F181" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G181" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36733,7 +37095,9 @@
       <c r="C182" s="2"/>
       <c r="D182" s="2"/>
       <c r="E182" s="2"/>
-      <c r="F182" s="1"/>
+      <c r="F182" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G182" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36750,7 +37114,9 @@
       <c r="C183" s="2"/>
       <c r="D183" s="2"/>
       <c r="E183" s="2"/>
-      <c r="F183" s="1"/>
+      <c r="F183" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G183" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36767,7 +37133,9 @@
       <c r="C184" s="2"/>
       <c r="D184" s="2"/>
       <c r="E184" s="2"/>
-      <c r="F184" s="1"/>
+      <c r="F184" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G184" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36784,7 +37152,9 @@
       <c r="C185" s="2"/>
       <c r="D185" s="2"/>
       <c r="E185" s="2"/>
-      <c r="F185" s="1"/>
+      <c r="F185" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G185" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36801,7 +37171,9 @@
       <c r="C186" s="2"/>
       <c r="D186" s="2"/>
       <c r="E186" s="2"/>
-      <c r="F186" s="1"/>
+      <c r="F186" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G186" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36818,7 +37190,9 @@
       <c r="C187" s="2"/>
       <c r="D187" s="2"/>
       <c r="E187" s="2"/>
-      <c r="F187" s="1"/>
+      <c r="F187" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G187" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36835,7 +37209,9 @@
       <c r="C188" s="2"/>
       <c r="D188" s="2"/>
       <c r="E188" s="2"/>
-      <c r="F188" s="1"/>
+      <c r="F188" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G188" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36852,7 +37228,9 @@
       <c r="C189" s="2"/>
       <c r="D189" s="2"/>
       <c r="E189" s="2"/>
-      <c r="F189" s="1"/>
+      <c r="F189" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G189" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36869,7 +37247,9 @@
       <c r="C190" s="2"/>
       <c r="D190" s="2"/>
       <c r="E190" s="2"/>
-      <c r="F190" s="1"/>
+      <c r="F190" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G190" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36886,7 +37266,9 @@
       <c r="C191" s="2"/>
       <c r="D191" s="2"/>
       <c r="E191" s="2"/>
-      <c r="F191" s="1"/>
+      <c r="F191" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G191" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36903,7 +37285,9 @@
       <c r="C192" s="2"/>
       <c r="D192" s="2"/>
       <c r="E192" s="2"/>
-      <c r="F192" s="1"/>
+      <c r="F192" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G192" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36920,7 +37304,9 @@
       <c r="C193" s="2"/>
       <c r="D193" s="2"/>
       <c r="E193" s="2"/>
-      <c r="F193" s="1"/>
+      <c r="F193" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G193" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36937,7 +37323,9 @@
       <c r="C194" s="2"/>
       <c r="D194" s="2"/>
       <c r="E194" s="2"/>
-      <c r="F194" s="1"/>
+      <c r="F194" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G194" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36954,7 +37342,9 @@
       <c r="C195" s="2"/>
       <c r="D195" s="2"/>
       <c r="E195" s="2"/>
-      <c r="F195" s="1"/>
+      <c r="F195" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G195" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36971,7 +37361,9 @@
       <c r="C196" s="2"/>
       <c r="D196" s="2"/>
       <c r="E196" s="2"/>
-      <c r="F196" s="1"/>
+      <c r="F196" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G196" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -36988,7 +37380,9 @@
       <c r="C197" s="2"/>
       <c r="D197" s="2"/>
       <c r="E197" s="2"/>
-      <c r="F197" s="1"/>
+      <c r="F197" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G197" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -37005,7 +37399,9 @@
       <c r="C198" s="2"/>
       <c r="D198" s="2"/>
       <c r="E198" s="2"/>
-      <c r="F198" s="1"/>
+      <c r="F198" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G198" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -37022,7 +37418,9 @@
       <c r="C199" s="2"/>
       <c r="D199" s="2"/>
       <c r="E199" s="2"/>
-      <c r="F199" s="1"/>
+      <c r="F199" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G199" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>
@@ -37039,7 +37437,9 @@
       <c r="C200" s="2"/>
       <c r="D200" s="2"/>
       <c r="E200" s="2"/>
-      <c r="F200" s="1"/>
+      <c r="F200" s="1">
+        <f t="shared" si="0"/>
+      </c>
       <c r="G200" s="1">
         <f>MAX(0,tblGoals[[#This Row],[Target Amount]]-tblGoals[[#This Row],[Current Saved Amount]])</f>
         <v>0</v>

</xml_diff>

<commit_message>
feat(liability-engine): complete T007 liability engine integration
</commit_message>
<xml_diff>
--- a/workbook/FinanceOS_v1.0.xlsx
+++ b/workbook/FinanceOS_v1.0.xlsx
@@ -79,6 +79,7 @@
     <definedName name="valPriority">Helpers!$B$139</definedName>
     <definedName name="valThemes">Helpers!$B$142</definedName>
     <definedName name="valTransactionTypes">Helpers!$B$145</definedName>
+    <definedName name="outLiabilityPaymentTotal">'Business Engine'!$B$46</definedName>
   </definedNames>
   <calcPr calcId="181029" forceFullCalc="1"/>
   <extLst>
@@ -90,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="358">
   <si>
     <t>Setting ID</t>
   </si>
@@ -1162,6 +1163,9 @@
   <si>
     <t>valBlank</t>
   </si>
+  <si>
+    <t>Liability Payment Total</t>
+  </si>
 </sst>
 </file>
 
@@ -5825,7 +5829,7 @@
         <v>257</v>
       </c>
       <c r="B42" s="1">
-        <f>IFERROR(SUMIFS(tblLiabilities[Outstanding Balance],tblLiabilities[Status],"Active"),0)</f>
+        <f>IFERROR(MAX(0,SUMIFS(tblLiabilities[Outstanding Balance],tblLiabilities[Status],"Active")),0)</f>
         <v>0</v>
       </c>
       <c r="D42" s="1">
@@ -5969,6 +5973,13 @@
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="B46" s="1">
+        <f>SUM(SUMIFS(tblTransactions[Amount],tblTransactions[Destination Type],"Liability",tblTransactions[Transaction Type],{"Expense","Transfer"},tblTransactions[Transaction Status],"Completed"))+SUM(SUMIFS(tblTransactions[Amount],tblTransactions[Destination Type],"Liability",tblTransactions[Transaction Type],{"Expense","Transfer"},tblTransactions[Transaction Status],"Reconciled"))</f>
+        <v>0</v>
+      </c>
       <c r="D46" s="1">
         <f t="shared" si="0"/>
       </c>

</xml_diff>

<commit_message>
feat(asset-engine): complete T008 asset engine integration
</commit_message>
<xml_diff>
--- a/workbook/FinanceOS_v1.0.xlsx
+++ b/workbook/FinanceOS_v1.0.xlsx
@@ -80,6 +80,7 @@
     <definedName name="valThemes">Helpers!$B$142</definedName>
     <definedName name="valTransactionTypes">Helpers!$B$145</definedName>
     <definedName name="outLiabilityPaymentTotal">'Business Engine'!$B$46</definedName>
+    <definedName name="outAssetPurchaseTotal">'Business Engine'!$B$39</definedName>
   </definedNames>
   <calcPr calcId="181029" forceFullCalc="1"/>
   <extLst>
@@ -91,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="366">
   <si>
     <t>Setting ID</t>
   </si>
@@ -1166,6 +1167,30 @@
   <si>
     <t>Liability Payment Total</t>
   </si>
+  <si>
+    <t>Asset Purchase Total</t>
+  </si>
+  <si>
+    <t>Asset Category Totals</t>
+  </si>
+  <si>
+    <t>Investment Value</t>
+  </si>
+  <si>
+    <t>Physical Asset Value</t>
+  </si>
+  <si>
+    <t>Property Value</t>
+  </si>
+  <si>
+    <t>Retirement Asset Value</t>
+  </si>
+  <si>
+    <t>Cash Equivalent Value</t>
+  </si>
+  <si>
+    <t>Other Asset Value</t>
+  </si>
 </sst>
 </file>
 
@@ -1223,7 +1248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
@@ -1255,6 +1280,7 @@
     <xf numFmtId="167" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5122,7 +5148,7 @@
         <v>240</v>
       </c>
       <c r="B22" s="1">
-        <f>IFERROR(SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))+SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1)),0)</f>
+        <f>IFERROR(SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))+SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))-SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))-SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1)),0)</f>
         <v>0</v>
       </c>
       <c r="D22" s="1">
@@ -5159,7 +5185,7 @@
         <v>241</v>
       </c>
       <c r="B23" s="1">
-        <f>IFERROR(SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1)-1,1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1),1))+SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1)-1,1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1),1)),0)</f>
+        <f>IFERROR(SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1)-1,1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1),1))+SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1)-1,1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1),1))-SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1)-1,1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1),1))-SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1)-1,1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1),1)),0)</f>
         <v>0</v>
       </c>
       <c r="D23" s="1">
@@ -5196,7 +5222,7 @@
         <v>242</v>
       </c>
       <c r="B24" s="1">
-        <f>IFERROR(SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),1,1),tblTransactions[Transaction Date],"&lt;="&amp;$B$1)+SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),1,1),tblTransactions[Transaction Date],"&lt;="&amp;$B$1),0)</f>
+        <f>IFERROR(SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),1,1),tblTransactions[Transaction Date],"&lt;="&amp;$B$1)+SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),1,1),tblTransactions[Transaction Date],"&lt;="&amp;$B$1)-SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),1,1),tblTransactions[Transaction Date],"&lt;="&amp;$B$1)-SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),1,1),tblTransactions[Transaction Date],"&lt;="&amp;$B$1),0)</f>
         <v>0</v>
       </c>
       <c r="D24" s="1">
@@ -5233,7 +5259,7 @@
         <v>243</v>
       </c>
       <c r="B25" s="1">
-        <f>COUNTIFS(tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))+COUNTIFS(tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))</f>
+        <f>COUNTIFS(tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))+COUNTIFS(tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))-COUNTIFS(tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Completed",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))-COUNTIFS(tblTransactions[Transaction Type],"Expense",tblTransactions[Transaction Status],"Reconciled",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Date],"&gt;="&amp;DATE(YEAR($B$1),MONTH($B$1),1),tblTransactions[Transaction Date],"&lt;"&amp;DATE(YEAR($B$1),MONTH($B$1)+1,1))</f>
         <v>0</v>
       </c>
       <c r="D25" s="1">
@@ -5725,6 +5751,13 @@
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B39" s="1">
+        <f>IFERROR(SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Status],"Completed")+SUMIFS(tblTransactions[Amount],tblTransactions[Transaction Type],"Expense",tblTransactions[Destination Type],"Asset",tblTransactions[Transaction Status],"Reconciled"),0)</f>
+        <v>0</v>
+      </c>
       <c r="D39" s="1">
         <f t="shared" si="0"/>
       </c>
@@ -6798,6 +6831,9 @@
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
+        <v>359</v>
+      </c>
       <c r="D69" s="1">
         <f t="shared" si="0"/>
       </c>
@@ -6828,6 +6864,13 @@
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="B70" s="1">
+        <f>IFERROR(SUMIFS(tblAssets[Current Value],tblAssets[Status],"Active",tblAssets[Asset Category],"Investment"),0)</f>
+        <v>0</v>
+      </c>
       <c r="D70" s="1">
         <f t="shared" si="0"/>
       </c>
@@ -6858,6 +6901,13 @@
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A71" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="B71" s="1">
+        <f>IFERROR(SUMIFS(tblAssets[Current Value],tblAssets[Status],"Active",tblAssets[Asset Category],"Physical Asset"),0)</f>
+        <v>0</v>
+      </c>
       <c r="D71" s="1">
         <f t="shared" si="0"/>
       </c>
@@ -6888,6 +6938,13 @@
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B72" s="1">
+        <f>IFERROR(SUMIFS(tblAssets[Current Value],tblAssets[Status],"Active",tblAssets[Asset Category],"Property"),0)</f>
+        <v>0</v>
+      </c>
       <c r="D72" s="1">
         <f t="shared" si="0"/>
       </c>
@@ -6918,6 +6975,13 @@
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B73" s="1">
+        <f>IFERROR(SUMIFS(tblAssets[Current Value],tblAssets[Status],"Active",tblAssets[Asset Category],"Retirement Asset"),0)</f>
+        <v>0</v>
+      </c>
       <c r="D73" s="1">
         <f t="shared" si="0"/>
       </c>
@@ -6948,6 +7012,13 @@
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B74" s="1">
+        <f>IFERROR(SUMIFS(tblAssets[Current Value],tblAssets[Status],"Active",tblAssets[Asset Category],"Cash Equivalent"),0)</f>
+        <v>0</v>
+      </c>
       <c r="D74" s="1">
         <f t="shared" si="0"/>
       </c>
@@ -6978,6 +7049,13 @@
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A75" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B75" s="1">
+        <f>IFERROR(SUMIFS(tblAssets[Current Value],tblAssets[Status],"Active",tblAssets[Asset Category],"Other Asset"),0)</f>
+        <v>0</v>
+      </c>
       <c r="D75" s="1">
         <f t="shared" si="0"/>
       </c>
@@ -19326,11 +19404,11 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J2" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J2" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K2" s="2"/>
@@ -19347,11 +19425,11 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J3" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J3" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K3" s="2"/>
@@ -19368,11 +19446,11 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J4" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K4" s="2"/>
@@ -19389,11 +19467,11 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K5" s="2"/>
@@ -19410,11 +19488,11 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J6" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K6" s="2"/>
@@ -19431,11 +19509,11 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K7" s="2"/>
@@ -19452,11 +19530,11 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K8" s="2"/>
@@ -19473,11 +19551,11 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J9" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K9" s="2"/>
@@ -19494,11 +19572,11 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K10" s="2"/>
@@ -19515,11 +19593,11 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K11" s="2"/>
@@ -19536,11 +19614,11 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K12" s="2"/>
@@ -19557,11 +19635,11 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J13" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K13" s="2"/>
@@ -19578,11 +19656,11 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J14" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J14" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K14" s="2"/>
@@ -19599,11 +19677,11 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K15" s="2"/>
@@ -19620,11 +19698,11 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K16" s="2"/>
@@ -19641,11 +19719,11 @@
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J17" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K17" s="2"/>
@@ -19662,11 +19740,11 @@
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J18" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K18" s="2"/>
@@ -19683,11 +19761,11 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J19" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K19" s="2"/>
@@ -19704,11 +19782,11 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K20" s="2"/>
@@ -19725,11 +19803,11 @@
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J21" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K21" s="2"/>
@@ -19746,11 +19824,11 @@
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J22" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K22" s="2"/>
@@ -19767,11 +19845,11 @@
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K23" s="2"/>
@@ -19788,11 +19866,11 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J24" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K24" s="2"/>
@@ -19809,11 +19887,11 @@
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J25" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J25" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K25" s="2"/>
@@ -19830,11 +19908,11 @@
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J26" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J26" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K26" s="2"/>
@@ -19851,11 +19929,11 @@
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J27" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K27" s="2"/>
@@ -19872,11 +19950,11 @@
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J28" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J28" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K28" s="2"/>
@@ -19893,11 +19971,11 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J29" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J29" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K29" s="2"/>
@@ -19914,11 +19992,11 @@
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J30" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K30" s="2"/>
@@ -19935,11 +20013,11 @@
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J31" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K31" s="2"/>
@@ -19956,11 +20034,11 @@
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J32" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K32" s="2"/>
@@ -19977,11 +20055,11 @@
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J33" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J33" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K33" s="2"/>
@@ -19998,11 +20076,11 @@
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J34" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J34" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K34" s="2"/>
@@ -20019,11 +20097,11 @@
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J35" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K35" s="2"/>
@@ -20040,11 +20118,11 @@
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J36" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J36" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K36" s="2"/>
@@ -20061,11 +20139,11 @@
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J37" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K37" s="2"/>
@@ -20082,11 +20160,11 @@
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J38" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J38" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K38" s="2"/>
@@ -20103,11 +20181,11 @@
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J39" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J39" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K39" s="2"/>
@@ -20124,11 +20202,11 @@
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
       <c r="I40" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J40" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J40" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K40" s="2"/>
@@ -20145,11 +20223,11 @@
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
       <c r="I41" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J41" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J41" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K41" s="2"/>
@@ -20166,11 +20244,11 @@
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J42" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J42" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K42" s="2"/>
@@ -20187,11 +20265,11 @@
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J43" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J43" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K43" s="2"/>
@@ -20208,11 +20286,11 @@
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J44" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J44" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K44" s="2"/>
@@ -20229,11 +20307,11 @@
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
       <c r="I45" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J45" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J45" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K45" s="2"/>
@@ -20250,11 +20328,11 @@
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="I46" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J46" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J46" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K46" s="2"/>
@@ -20271,11 +20349,11 @@
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
       <c r="I47" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J47" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J47" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K47" s="2"/>
@@ -20292,11 +20370,11 @@
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
       <c r="I48" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J48" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J48" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K48" s="2"/>
@@ -20313,11 +20391,11 @@
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
       <c r="I49" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J49" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J49" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K49" s="2"/>
@@ -20334,11 +20412,11 @@
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
       <c r="I50" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J50" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J50" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K50" s="2"/>
@@ -20355,11 +20433,11 @@
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
       <c r="I51" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J51" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J51" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K51" s="2"/>
@@ -20376,11 +20454,11 @@
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
       <c r="I52" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J52" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J52" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K52" s="2"/>
@@ -20397,11 +20475,11 @@
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J53" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J53" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K53" s="2"/>
@@ -20418,11 +20496,11 @@
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="I54" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J54" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J54" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K54" s="2"/>
@@ -20439,11 +20517,11 @@
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="I55" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J55" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J55" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K55" s="2"/>
@@ -20460,11 +20538,11 @@
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J56" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J56" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K56" s="2"/>
@@ -20481,11 +20559,11 @@
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J57" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J57" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K57" s="2"/>
@@ -20502,11 +20580,11 @@
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J58" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J58" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K58" s="2"/>
@@ -20523,11 +20601,11 @@
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
       <c r="I59" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J59" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J59" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K59" s="2"/>
@@ -20544,11 +20622,11 @@
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
       <c r="I60" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J60" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J60" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K60" s="2"/>
@@ -20565,11 +20643,11 @@
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
       <c r="I61" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J61" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J61" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K61" s="2"/>
@@ -20586,11 +20664,11 @@
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
       <c r="I62" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J62" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J62" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K62" s="2"/>
@@ -20607,11 +20685,11 @@
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J63" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J63" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K63" s="2"/>
@@ -20628,11 +20706,11 @@
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
       <c r="I64" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J64" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J64" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K64" s="2"/>
@@ -20649,11 +20727,11 @@
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
       <c r="I65" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J65" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J65" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K65" s="2"/>
@@ -20670,11 +20748,11 @@
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
       <c r="I66" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J66" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J66" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K66" s="2"/>
@@ -20691,11 +20769,11 @@
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
       <c r="I67" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J67" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J67" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K67" s="2"/>
@@ -20712,11 +20790,11 @@
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
       <c r="I68" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J68" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J68" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K68" s="2"/>
@@ -20733,11 +20811,11 @@
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
       <c r="I69" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J69" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J69" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K69" s="2"/>
@@ -20754,11 +20832,11 @@
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
       <c r="I70" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J70" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J70" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K70" s="2"/>
@@ -20775,11 +20853,11 @@
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J71" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J71" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K71" s="2"/>
@@ -20796,11 +20874,11 @@
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J72" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J72" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K72" s="2"/>
@@ -20817,11 +20895,11 @@
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J73" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J73" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K73" s="2"/>
@@ -20838,11 +20916,11 @@
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J74" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J74" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K74" s="2"/>
@@ -20859,11 +20937,11 @@
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
       <c r="I75" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J75" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J75" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K75" s="2"/>
@@ -20880,11 +20958,11 @@
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J76" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J76" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K76" s="2"/>
@@ -20901,11 +20979,11 @@
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J77" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J77" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K77" s="2"/>
@@ -20922,11 +21000,11 @@
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J78" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J78" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K78" s="2"/>
@@ -20943,11 +21021,11 @@
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J79" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J79" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K79" s="2"/>
@@ -20964,11 +21042,11 @@
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J80" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J80" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K80" s="2"/>
@@ -20985,11 +21063,11 @@
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
       <c r="I81" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J81" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J81" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K81" s="2"/>
@@ -21006,11 +21084,11 @@
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
       <c r="I82" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J82" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J82" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K82" s="2"/>
@@ -21027,11 +21105,11 @@
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
       <c r="I83" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J83" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J83" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K83" s="2"/>
@@ -21048,11 +21126,11 @@
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
       <c r="I84" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J84" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J84" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K84" s="2"/>
@@ -21069,11 +21147,11 @@
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
       <c r="I85" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J85" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J85" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K85" s="2"/>
@@ -21090,11 +21168,11 @@
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
       <c r="I86" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J86" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J86" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K86" s="2"/>
@@ -21111,11 +21189,11 @@
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
       <c r="I87" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J87" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J87" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K87" s="2"/>
@@ -21132,11 +21210,11 @@
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
       <c r="I88" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J88" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J88" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K88" s="2"/>
@@ -21153,11 +21231,11 @@
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
       <c r="I89" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J89" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J89" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K89" s="2"/>
@@ -21174,11 +21252,11 @@
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
       <c r="I90" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J90" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J90" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K90" s="2"/>
@@ -21195,11 +21273,11 @@
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
       <c r="I91" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J91" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J91" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K91" s="2"/>
@@ -21216,11 +21294,11 @@
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
       <c r="I92" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J92" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J92" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K92" s="2"/>
@@ -21237,11 +21315,11 @@
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
       <c r="I93" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J93" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J93" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K93" s="2"/>
@@ -21258,11 +21336,11 @@
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
       <c r="I94" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J94" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J94" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K94" s="2"/>
@@ -21279,11 +21357,11 @@
       <c r="G95" s="2"/>
       <c r="H95" s="2"/>
       <c r="I95" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J95" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J95" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K95" s="2"/>
@@ -21300,11 +21378,11 @@
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
       <c r="I96" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J96" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J96" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K96" s="2"/>
@@ -21321,11 +21399,11 @@
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
       <c r="I97" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J97" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J97" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K97" s="2"/>
@@ -21342,11 +21420,11 @@
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
       <c r="I98" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J98" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J98" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K98" s="2"/>
@@ -21363,11 +21441,11 @@
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
       <c r="I99" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J99" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J99" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K99" s="2"/>
@@ -21384,11 +21462,11 @@
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
       <c r="I100" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J100" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J100" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K100" s="2"/>
@@ -21405,11 +21483,11 @@
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
       <c r="I101" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J101" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J101" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K101" s="2"/>
@@ -21426,11 +21504,11 @@
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
       <c r="I102" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J102" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J102" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K102" s="2"/>
@@ -21447,11 +21525,11 @@
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
       <c r="I103" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J103" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J103" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K103" s="2"/>
@@ -21468,11 +21546,11 @@
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
       <c r="I104" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J104" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J104" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K104" s="2"/>
@@ -21489,11 +21567,11 @@
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
       <c r="I105" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J105" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J105" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K105" s="2"/>
@@ -21510,11 +21588,11 @@
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
       <c r="I106" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J106" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J106" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K106" s="2"/>
@@ -21531,11 +21609,11 @@
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
       <c r="I107" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J107" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J107" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K107" s="2"/>
@@ -21552,11 +21630,11 @@
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
       <c r="I108" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J108" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J108" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K108" s="2"/>
@@ -21573,11 +21651,11 @@
       <c r="G109" s="2"/>
       <c r="H109" s="2"/>
       <c r="I109" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J109" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J109" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K109" s="2"/>
@@ -21594,11 +21672,11 @@
       <c r="G110" s="2"/>
       <c r="H110" s="2"/>
       <c r="I110" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J110" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J110" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K110" s="2"/>
@@ -21615,11 +21693,11 @@
       <c r="G111" s="2"/>
       <c r="H111" s="2"/>
       <c r="I111" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J111" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J111" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K111" s="2"/>
@@ -21636,11 +21714,11 @@
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
       <c r="I112" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J112" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J112" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K112" s="2"/>
@@ -21657,11 +21735,11 @@
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
       <c r="I113" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J113" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J113" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K113" s="2"/>
@@ -21678,11 +21756,11 @@
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
       <c r="I114" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J114" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J114" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K114" s="2"/>
@@ -21699,11 +21777,11 @@
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
       <c r="I115" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J115" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J115" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K115" s="2"/>
@@ -21720,11 +21798,11 @@
       <c r="G116" s="2"/>
       <c r="H116" s="2"/>
       <c r="I116" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J116" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J116" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K116" s="2"/>
@@ -21741,11 +21819,11 @@
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
       <c r="I117" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J117" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J117" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K117" s="2"/>
@@ -21762,11 +21840,11 @@
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
       <c r="I118" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J118" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J118" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K118" s="2"/>
@@ -21783,11 +21861,11 @@
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
       <c r="I119" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J119" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J119" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K119" s="2"/>
@@ -21804,11 +21882,11 @@
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
       <c r="I120" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J120" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J120" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K120" s="2"/>
@@ -21825,11 +21903,11 @@
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
       <c r="I121" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J121" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J121" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K121" s="2"/>
@@ -21846,11 +21924,11 @@
       <c r="G122" s="2"/>
       <c r="H122" s="2"/>
       <c r="I122" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J122" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J122" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K122" s="2"/>
@@ -21867,11 +21945,11 @@
       <c r="G123" s="2"/>
       <c r="H123" s="2"/>
       <c r="I123" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J123" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J123" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K123" s="2"/>
@@ -21888,11 +21966,11 @@
       <c r="G124" s="2"/>
       <c r="H124" s="2"/>
       <c r="I124" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J124" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J124" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K124" s="2"/>
@@ -21909,11 +21987,11 @@
       <c r="G125" s="2"/>
       <c r="H125" s="2"/>
       <c r="I125" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J125" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J125" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K125" s="2"/>
@@ -21930,11 +22008,11 @@
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
       <c r="I126" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J126" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J126" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K126" s="2"/>
@@ -21951,11 +22029,11 @@
       <c r="G127" s="2"/>
       <c r="H127" s="2"/>
       <c r="I127" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J127" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J127" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K127" s="2"/>
@@ -21972,11 +22050,11 @@
       <c r="G128" s="2"/>
       <c r="H128" s="2"/>
       <c r="I128" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J128" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J128" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K128" s="2"/>
@@ -21993,11 +22071,11 @@
       <c r="G129" s="2"/>
       <c r="H129" s="2"/>
       <c r="I129" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J129" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J129" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K129" s="2"/>
@@ -22014,11 +22092,11 @@
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
       <c r="I130" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J130" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J130" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K130" s="2"/>
@@ -22035,11 +22113,11 @@
       <c r="G131" s="2"/>
       <c r="H131" s="2"/>
       <c r="I131" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J131" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J131" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K131" s="2"/>
@@ -22056,11 +22134,11 @@
       <c r="G132" s="2"/>
       <c r="H132" s="2"/>
       <c r="I132" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J132" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J132" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K132" s="2"/>
@@ -22077,11 +22155,11 @@
       <c r="G133" s="2"/>
       <c r="H133" s="2"/>
       <c r="I133" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J133" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J133" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K133" s="2"/>
@@ -22098,11 +22176,11 @@
       <c r="G134" s="2"/>
       <c r="H134" s="2"/>
       <c r="I134" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J134" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J134" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K134" s="2"/>
@@ -22119,11 +22197,11 @@
       <c r="G135" s="2"/>
       <c r="H135" s="2"/>
       <c r="I135" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J135" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J135" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K135" s="2"/>
@@ -22140,11 +22218,11 @@
       <c r="G136" s="2"/>
       <c r="H136" s="2"/>
       <c r="I136" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J136" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J136" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K136" s="2"/>
@@ -22161,11 +22239,11 @@
       <c r="G137" s="2"/>
       <c r="H137" s="2"/>
       <c r="I137" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J137" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J137" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K137" s="2"/>
@@ -22182,11 +22260,11 @@
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
       <c r="I138" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J138" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J138" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K138" s="2"/>
@@ -22203,11 +22281,11 @@
       <c r="G139" s="2"/>
       <c r="H139" s="2"/>
       <c r="I139" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J139" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J139" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K139" s="2"/>
@@ -22224,11 +22302,11 @@
       <c r="G140" s="2"/>
       <c r="H140" s="2"/>
       <c r="I140" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J140" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J140" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K140" s="2"/>
@@ -22245,11 +22323,11 @@
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
       <c r="I141" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J141" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J141" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K141" s="2"/>
@@ -22266,11 +22344,11 @@
       <c r="G142" s="2"/>
       <c r="H142" s="2"/>
       <c r="I142" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J142" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J142" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K142" s="2"/>
@@ -22287,11 +22365,11 @@
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
       <c r="I143" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J143" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J143" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K143" s="2"/>
@@ -22308,11 +22386,11 @@
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
       <c r="I144" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J144" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J144" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K144" s="2"/>
@@ -22329,11 +22407,11 @@
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
       <c r="I145" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J145" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J145" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K145" s="2"/>
@@ -22350,11 +22428,11 @@
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
       <c r="I146" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J146" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J146" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K146" s="2"/>
@@ -22371,11 +22449,11 @@
       <c r="G147" s="2"/>
       <c r="H147" s="2"/>
       <c r="I147" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J147" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J147" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K147" s="2"/>
@@ -22392,11 +22470,11 @@
       <c r="G148" s="2"/>
       <c r="H148" s="2"/>
       <c r="I148" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J148" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J148" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K148" s="2"/>
@@ -22413,11 +22491,11 @@
       <c r="G149" s="2"/>
       <c r="H149" s="2"/>
       <c r="I149" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J149" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J149" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K149" s="2"/>
@@ -22434,11 +22512,11 @@
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
       <c r="I150" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J150" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J150" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K150" s="2"/>
@@ -22455,11 +22533,11 @@
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
       <c r="I151" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J151" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J151" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K151" s="2"/>
@@ -22476,11 +22554,11 @@
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
       <c r="I152" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J152" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J152" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K152" s="2"/>
@@ -22497,11 +22575,11 @@
       <c r="G153" s="2"/>
       <c r="H153" s="2"/>
       <c r="I153" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J153" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J153" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K153" s="2"/>
@@ -22518,11 +22596,11 @@
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
       <c r="I154" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J154" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J154" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K154" s="2"/>
@@ -22539,11 +22617,11 @@
       <c r="G155" s="2"/>
       <c r="H155" s="2"/>
       <c r="I155" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J155" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J155" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K155" s="2"/>
@@ -22560,11 +22638,11 @@
       <c r="G156" s="2"/>
       <c r="H156" s="2"/>
       <c r="I156" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J156" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J156" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K156" s="2"/>
@@ -22581,11 +22659,11 @@
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
       <c r="I157" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J157" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J157" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K157" s="2"/>
@@ -22602,11 +22680,11 @@
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
       <c r="I158" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J158" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J158" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K158" s="2"/>
@@ -22623,11 +22701,11 @@
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
       <c r="I159" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J159" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J159" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K159" s="2"/>
@@ -22644,11 +22722,11 @@
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
       <c r="I160" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J160" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J160" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K160" s="2"/>
@@ -22665,11 +22743,11 @@
       <c r="G161" s="2"/>
       <c r="H161" s="2"/>
       <c r="I161" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J161" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J161" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K161" s="2"/>
@@ -22686,11 +22764,11 @@
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
       <c r="I162" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J162" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J162" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K162" s="2"/>
@@ -22707,11 +22785,11 @@
       <c r="G163" s="2"/>
       <c r="H163" s="2"/>
       <c r="I163" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J163" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J163" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K163" s="2"/>
@@ -22728,11 +22806,11 @@
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
       <c r="I164" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J164" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J164" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K164" s="2"/>
@@ -22749,11 +22827,11 @@
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
       <c r="I165" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J165" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J165" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K165" s="2"/>
@@ -22770,11 +22848,11 @@
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
       <c r="I166" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J166" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J166" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K166" s="2"/>
@@ -22791,11 +22869,11 @@
       <c r="G167" s="2"/>
       <c r="H167" s="2"/>
       <c r="I167" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J167" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J167" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K167" s="2"/>
@@ -22812,11 +22890,11 @@
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
       <c r="I168" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J168" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J168" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K168" s="2"/>
@@ -22833,11 +22911,11 @@
       <c r="G169" s="2"/>
       <c r="H169" s="2"/>
       <c r="I169" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J169" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J169" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K169" s="2"/>
@@ -22854,11 +22932,11 @@
       <c r="G170" s="2"/>
       <c r="H170" s="2"/>
       <c r="I170" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J170" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J170" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K170" s="2"/>
@@ -22875,11 +22953,11 @@
       <c r="G171" s="2"/>
       <c r="H171" s="2"/>
       <c r="I171" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J171" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J171" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K171" s="2"/>
@@ -22896,11 +22974,11 @@
       <c r="G172" s="2"/>
       <c r="H172" s="2"/>
       <c r="I172" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J172" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J172" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K172" s="2"/>
@@ -22917,11 +22995,11 @@
       <c r="G173" s="2"/>
       <c r="H173" s="2"/>
       <c r="I173" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J173" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J173" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K173" s="2"/>
@@ -22938,11 +23016,11 @@
       <c r="G174" s="2"/>
       <c r="H174" s="2"/>
       <c r="I174" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J174" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J174" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K174" s="2"/>
@@ -22959,11 +23037,11 @@
       <c r="G175" s="2"/>
       <c r="H175" s="2"/>
       <c r="I175" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J175" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J175" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K175" s="2"/>
@@ -22980,11 +23058,11 @@
       <c r="G176" s="2"/>
       <c r="H176" s="2"/>
       <c r="I176" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J176" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J176" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K176" s="2"/>
@@ -23001,11 +23079,11 @@
       <c r="G177" s="2"/>
       <c r="H177" s="2"/>
       <c r="I177" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J177" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J177" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K177" s="2"/>
@@ -23022,11 +23100,11 @@
       <c r="G178" s="2"/>
       <c r="H178" s="2"/>
       <c r="I178" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J178" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J178" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K178" s="2"/>
@@ -23043,11 +23121,11 @@
       <c r="G179" s="2"/>
       <c r="H179" s="2"/>
       <c r="I179" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J179" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J179" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K179" s="2"/>
@@ -23064,11 +23142,11 @@
       <c r="G180" s="2"/>
       <c r="H180" s="2"/>
       <c r="I180" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J180" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J180" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K180" s="2"/>
@@ -23085,11 +23163,11 @@
       <c r="G181" s="2"/>
       <c r="H181" s="2"/>
       <c r="I181" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J181" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J181" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K181" s="2"/>
@@ -23106,11 +23184,11 @@
       <c r="G182" s="2"/>
       <c r="H182" s="2"/>
       <c r="I182" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J182" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J182" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K182" s="2"/>
@@ -23127,11 +23205,11 @@
       <c r="G183" s="2"/>
       <c r="H183" s="2"/>
       <c r="I183" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J183" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J183" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K183" s="2"/>
@@ -23148,11 +23226,11 @@
       <c r="G184" s="2"/>
       <c r="H184" s="2"/>
       <c r="I184" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J184" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J184" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K184" s="2"/>
@@ -23169,11 +23247,11 @@
       <c r="G185" s="2"/>
       <c r="H185" s="2"/>
       <c r="I185" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J185" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J185" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K185" s="2"/>
@@ -23190,11 +23268,11 @@
       <c r="G186" s="2"/>
       <c r="H186" s="2"/>
       <c r="I186" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J186" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J186" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K186" s="2"/>
@@ -23211,11 +23289,11 @@
       <c r="G187" s="2"/>
       <c r="H187" s="2"/>
       <c r="I187" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J187" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J187" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K187" s="2"/>
@@ -23232,11 +23310,11 @@
       <c r="G188" s="2"/>
       <c r="H188" s="2"/>
       <c r="I188" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J188" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J188" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K188" s="2"/>
@@ -23253,11 +23331,11 @@
       <c r="G189" s="2"/>
       <c r="H189" s="2"/>
       <c r="I189" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J189" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J189" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K189" s="2"/>
@@ -23274,11 +23352,11 @@
       <c r="G190" s="2"/>
       <c r="H190" s="2"/>
       <c r="I190" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J190" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J190" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K190" s="2"/>
@@ -23295,11 +23373,11 @@
       <c r="G191" s="2"/>
       <c r="H191" s="2"/>
       <c r="I191" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J191" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J191" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K191" s="2"/>
@@ -23316,11 +23394,11 @@
       <c r="G192" s="2"/>
       <c r="H192" s="2"/>
       <c r="I192" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J192" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J192" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K192" s="2"/>
@@ -23337,11 +23415,11 @@
       <c r="G193" s="2"/>
       <c r="H193" s="2"/>
       <c r="I193" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J193" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J193" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K193" s="2"/>
@@ -23358,11 +23436,11 @@
       <c r="G194" s="2"/>
       <c r="H194" s="2"/>
       <c r="I194" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J194" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J194" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K194" s="2"/>
@@ -23379,11 +23457,11 @@
       <c r="G195" s="2"/>
       <c r="H195" s="2"/>
       <c r="I195" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J195" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J195" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K195" s="2"/>
@@ -23400,11 +23478,11 @@
       <c r="G196" s="2"/>
       <c r="H196" s="2"/>
       <c r="I196" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J196" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J196" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K196" s="2"/>
@@ -23421,11 +23499,11 @@
       <c r="G197" s="2"/>
       <c r="H197" s="2"/>
       <c r="I197" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J197" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J197" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K197" s="2"/>
@@ -23442,11 +23520,11 @@
       <c r="G198" s="2"/>
       <c r="H198" s="2"/>
       <c r="I198" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J198" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J198" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K198" s="2"/>
@@ -23463,11 +23541,11 @@
       <c r="G199" s="2"/>
       <c r="H199" s="2"/>
       <c r="I199" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J199" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J199" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K199" s="2"/>
@@ -23484,11 +23562,11 @@
       <c r="G200" s="2"/>
       <c r="H200" s="2"/>
       <c r="I200" s="1">
-        <f>tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]]</f>
-        <v>0</v>
-      </c>
-      <c r="J200" s="1">
-        <f>IFERROR(tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]],0)</f>
+        <f>IF(tblAssets[[#This Row],[Asset ID]]="","",tblAssets[[#This Row],[Current Value]]-tblAssets[[#This Row],[Purchase Value]])</f>
+        <v>0</v>
+      </c>
+      <c r="J200" s="11">
+        <f>IF(OR(tblAssets[[#This Row],[Asset ID]]="",tblAssets[[#This Row],[Purchase Value]]=0),"",tblAssets[[#This Row],[Appreciation Amount]]/tblAssets[[#This Row],[Purchase Value]])</f>
         <v>0</v>
       </c>
       <c r="K200" s="2"/>
@@ -23497,7 +23575,7 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" insertRows="0" deleteRows="0" sort="0" autoFilter="0"/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Select a value from the list." promptTitle="Select a value" prompt="Choose from the list." sqref="D2:D200" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>rngAssetType</formula1>
     </dataValidation>
@@ -23508,7 +23586,10 @@
       <formula1>rngOwnershipType</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Select a value from the list." promptTitle="Select a value" prompt="Choose from the list." sqref="L2:L200" xr:uid="{00000000-0002-0000-0400-000003000000}">
-      <formula1>rngAccountStatus</formula1>
+      <formula1>"Active,Sold"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Current Value" error="Current Value must be greater than or equal to 0." promptTitle="Current Value" prompt="Enter a value of 0 or greater." sqref="H2:H200">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(analysis-engine): implement RC1 financial health analysis section
</commit_message>
<xml_diff>
--- a/workbook/FinanceOS_v1.0.xlsx
+++ b/workbook/FinanceOS_v1.0.xlsx
@@ -81,6 +81,14 @@
     <definedName name="valTransactionTypes">Helpers!$B$145</definedName>
     <definedName name="outLiabilityPaymentTotal">'Business Engine'!$B$46</definedName>
     <definedName name="outAssetPurchaseTotal">'Business Engine'!$B$39</definedName>
+    <definedName name="analysisSavingsHealth">'Analysis Engine'!$B$158</definedName>
+    <definedName name="analysisExpenseHealth">'Analysis Engine'!$B$159</definedName>
+    <definedName name="analysisDebtHealth">'Analysis Engine'!$B$160</definedName>
+    <definedName name="analysisAssetHealth">'Analysis Engine'!$B$161</definedName>
+    <definedName name="analysisGoalHealth">'Analysis Engine'!$B$162</definedName>
+    <definedName name="analysisLiquidityHealth">'Analysis Engine'!$B$163</definedName>
+    <definedName name="analysisNetWorthHealth">'Analysis Engine'!$B$164</definedName>
+    <definedName name="analysisCashFlowHealth">'Analysis Engine'!$B$165</definedName>
   </definedNames>
   <calcPr calcId="181029" forceFullCalc="1"/>
   <extLst>
@@ -92,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="379">
   <si>
     <t>Setting ID</t>
   </si>
@@ -1190,6 +1198,45 @@
   </si>
   <si>
     <t>Other Asset Value</t>
+  </si>
+  <si>
+    <t>SECTION 10 — RC1 Analysis Health</t>
+  </si>
+  <si>
+    <t>Dimension</t>
+  </si>
+  <si>
+    <t>Band</t>
+  </si>
+  <si>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Savings Health</t>
+  </si>
+  <si>
+    <t>Expense Health</t>
+  </si>
+  <si>
+    <t>Debt Health</t>
+  </si>
+  <si>
+    <t>Asset Health</t>
+  </si>
+  <si>
+    <t>Goal Health</t>
+  </si>
+  <si>
+    <t>Liquidity Health</t>
+  </si>
+  <si>
+    <t>Net Worth Health</t>
+  </si>
+  <si>
+    <t>Cash Flow Health</t>
   </si>
 </sst>
 </file>
@@ -10844,7 +10891,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:AA154"/>
+  <dimension ref="A1:AA165"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -12739,6 +12786,161 @@
       <c r="B154" s="1">
         <f>IFERROR($B$127/$B$45,0)</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A156" s="1" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A157" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B157" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="D157" s="1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A158" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B158" s="1" t="str">
+        <f>LET(inc,'Business Engine'!$B$16,rate,'Business Engine'!$B$30,IF(inc=0,"Unavailable",IF(rate&lt;0,"Critical",IF(rate&lt;0.1,"Weak",IF(rate&lt;0.2,"Moderate",IF(rate&lt;0.3,"Strong","Excellent"))))))</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="C158" s="1" t="str">
+        <f>LET(b,B158,IF(b="Unavailable","",IF(b="Critical",0,IF(b="Weak",25,IF(b="Moderate",50,IF((b="Strong")+(b="Healthy"),75,IF(b="Excellent",100,"")))))))</f>
+        <v/>
+      </c>
+      <c r="D158" s="1" t="str">
+        <f>LET(b,B158,IF(b="Unavailable","",IF(b="Critical","Red",IF(b="Weak","Orange",IF(b="Moderate","Yellow",IF((b="Strong")+(b="Healthy"),"Green",IF(b="Excellent","Green","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A159" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B159" s="1" t="str">
+        <f>LET(inc,'Business Engine'!$B$16,exp,'Business Engine'!$B$22,IF(inc=0,IF(exp=0,"Unavailable",IF(exp&gt;0,"Critical",LET(ratio,exp/inc,IF(ratio&lt;0.5,"Excellent",IF(ratio&lt;0.7,"Strong",IF(ratio&lt;0.85,"Moderate",IF(ratio&lt;1,"Weak","Critical"))))))),LET(ratio,exp/inc,IF(ratio&lt;0.5,"Excellent",IF(ratio&lt;0.7,"Strong",IF(ratio&lt;0.85,"Moderate",IF(ratio&lt;1,"Weak","Critical")))))))</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="C159" s="1" t="str">
+        <f>LET(b,B159,IF(b="Unavailable","",IF(b="Critical",0,IF(b="Weak",25,IF(b="Moderate",50,IF((b="Strong")+(b="Healthy"),75,IF(b="Excellent",100,"")))))))</f>
+        <v/>
+      </c>
+      <c r="D159" s="1" t="str">
+        <f>LET(b,B159,IF(b="Unavailable","",IF(b="Critical","Red",IF(b="Weak","Orange",IF(b="Moderate","Yellow",IF((b="Strong")+(b="Healthy"),"Green",IF(b="Excellent","Green","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A160" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="B160" s="1" t="str">
+        <f>LET(b4,'Business Engine'!$B$4,b16,'Business Engine'!$B$16,b22,'Business Engine'!$B$22,b35,'Business Engine'!$B$35,b38,'Business Engine'!$B$38,b42,'Business Engine'!$B$42,b45,'Business Engine'!$B$45,b56,'Business Engine'!$B$56,b57,'Business Engine'!$B$57,emi,'Business Engine'!$B$66,emiBand,IF(emi&lt;0.15,"Excellent",IF(emi&lt;0.25,"Strong",IF(emi&lt;0.35,"Moderate",IF(emi&lt;0.5,"Weak","Critical")))),afterEmpty,IF(b45=0,IF(b42=0,"Excellent",emiBand),IF(b16=0,IF(b45&gt;0,"Critical",emiBand),emiBand)),IF(b4=0,IF(b16=0,IF(b22=0,IF(b35=0,IF(b38=0,IF(b42=0,IF(b45=0,IF(b56=0,IF(b57=0,"Unavailable",afterEmpty),afterEmpty),afterEmpty),afterEmpty),afterEmpty),afterEmpty),afterEmpty),afterEmpty),afterEmpty))</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="C160" s="1" t="str">
+        <f>LET(b,B160,IF(b="Unavailable","",IF(b="Critical",0,IF(b="Weak",25,IF(b="Moderate",50,IF((b="Strong")+(b="Healthy"),75,IF(b="Excellent",100,"")))))))</f>
+        <v/>
+      </c>
+      <c r="D160" s="1" t="str">
+        <f>LET(b,B160,IF(b="Unavailable","",IF(b="Critical","Red",IF(b="Weak","Orange",IF(b="Moderate","Yellow",IF((b="Strong")+(b="Healthy"),"Green",IF(b="Excellent","Green","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A161" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B161" s="1" t="str">
+        <f>LET(cnt,'Business Engine'!$B$38,tot,'Business Engine'!$B$35,cash,'Business Engine'!$B$74,den,tot-cash,IF(cnt=0,"Unavailable",IF(den&lt;=0,"Unavailable",LET(conc,MAX('Business Engine'!$B$70,'Business Engine'!$B$71,'Business Engine'!$B$72,'Business Engine'!$B$73,'Business Engine'!$B$75)/den,IF(conc&lt;=0.4,"Excellent",IF(conc&lt;=0.6,"Strong",IF(conc&lt;=0.8,"Moderate",IF(conc&lt;=0.95,"Weak","Critical"))))))))</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="C161" s="1" t="str">
+        <f>LET(b,B161,IF(b="Unavailable","",IF(b="Critical",0,IF(b="Weak",25,IF(b="Moderate",50,IF((b="Strong")+(b="Healthy"),75,IF(b="Excellent",100,"")))))))</f>
+        <v/>
+      </c>
+      <c r="D161" s="1" t="str">
+        <f>LET(b,B161,IF(b="Unavailable","",IF(b="Critical","Red",IF(b="Weak","Orange",IF(b="Moderate","Yellow",IF((b="Strong")+(b="Healthy"),"Green",IF(b="Excellent","Green","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A162" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="B162" s="1" t="str">
+        <f>LET(n,'Business Engine'!$B$56+'Business Engine'!$B$57,pct,'Business Engine'!$B$58,IF(n=0,"Unavailable",IF(pct&gt;=0.8,"Excellent",IF(pct&gt;=0.5,"Strong",IF(pct&gt;=0.25,"Moderate",IF(pct&gt;0,"Weak","Critical"))))))</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="C162" s="1" t="str">
+        <f>LET(b,B162,IF(b="Unavailable","",IF(b="Critical",0,IF(b="Weak",25,IF(b="Moderate",50,IF((b="Strong")+(b="Healthy"),75,IF(b="Excellent",100,"")))))))</f>
+        <v/>
+      </c>
+      <c r="D162" s="1" t="str">
+        <f>LET(b,B162,IF(b="Unavailable","",IF(b="Critical","Red",IF(b="Weak","Orange",IF(b="Moderate","Yellow",IF((b="Strong")+(b="Healthy"),"Green",IF(b="Excellent","Green","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A163" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B163" s="1" t="str">
+        <f>LET(cash,'Business Engine'!$B$4,exp,'Business Engine'!$B$22,IF(exp=0,IF(cash=0,"Unavailable",IF(cash&gt;0,"Excellent",LET(m,cash/exp,IF(m&lt;1,"Critical",IF(m&lt;3,"Weak",IF(m&lt;6,"Moderate",IF(m&lt;=12,"Healthy","Excellent"))))))),LET(m,cash/exp,IF(m&lt;1,"Critical",IF(m&lt;3,"Weak",IF(m&lt;6,"Moderate",IF(m&lt;=12,"Healthy","Excellent")))))))</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="C163" s="1" t="str">
+        <f>LET(b,B163,IF(b="Unavailable","",IF(b="Critical",0,IF(b="Weak",25,IF(b="Moderate",50,IF((b="Strong")+(b="Healthy"),75,IF(b="Excellent",100,"")))))))</f>
+        <v/>
+      </c>
+      <c r="D163" s="1" t="str">
+        <f>LET(b,B163,IF(b="Unavailable","",IF(b="Critical","Red",IF(b="Weak","Orange",IF(b="Moderate","Yellow",IF((b="Strong")+(b="Healthy"),"Green",IF(b="Excellent","Green","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A164" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B164" s="1" t="str">
+        <f>LET(b4,'Business Engine'!$B$4,b35,'Business Engine'!$B$35,b42,'Business Engine'!$B$42,nw,'Business Engine'!$B$48,lev,'Business Engine'!$B$68,nwBand,IF(nw&lt;0,"Critical",IF(nw=0,"Weak",IF(lev&gt;=0.7,"Weak",IF(lev&gt;=0.4,"Moderate",IF(lev&gt;=0.2,"Strong","Excellent"))))),IF(b4=0,IF(b35=0,IF(b42=0,"Unavailable",nwBand),nwBand),nwBand))</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="C164" s="1" t="str">
+        <f>LET(b,B164,IF(b="Unavailable","",IF(b="Critical",0,IF(b="Weak",25,IF(b="Moderate",50,IF((b="Strong")+(b="Healthy"),75,IF(b="Excellent",100,"")))))))</f>
+        <v/>
+      </c>
+      <c r="D164" s="1" t="str">
+        <f>LET(b,B164,IF(b="Unavailable","",IF(b="Critical","Red",IF(b="Weak","Orange",IF(b="Moderate","Yellow",IF((b="Strong")+(b="Healthy"),"Green",IF(b="Excellent","Green","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A165" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="B165" s="1" t="str">
+        <f>LET(inc,'Business Engine'!$B$16,exp,'Business Engine'!$B$22,sav,'Business Engine'!$B$29,IF(inc=0,IF(exp=0,"Unavailable",IF(exp&gt;0,"Critical",IF(sav&lt;0,"Critical",IF(sav=0,"Weak",LET(ratio,sav/inc,IF(ratio&lt;0.1,"Moderate",IF(ratio&lt;0.25,"Strong","Excellent"))))))),IF(sav&lt;0,"Critical",IF(sav=0,"Weak",LET(ratio,sav/inc,IF(ratio&lt;0.1,"Moderate",IF(ratio&lt;0.25,"Strong","Excellent")))))))</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="C165" s="1" t="str">
+        <f>LET(b,B165,IF(b="Unavailable","",IF(b="Critical",0,IF(b="Weak",25,IF(b="Moderate",50,IF((b="Strong")+(b="Healthy"),75,IF(b="Excellent",100,"")))))))</f>
+        <v/>
+      </c>
+      <c r="D165" s="1" t="str">
+        <f>LET(b,B165,IF(b="Unavailable","",IF(b="Critical","Red",IF(b="Weak","Orange",IF(b="Moderate","Yellow",IF((b="Strong")+(b="Healthy"),"Green",IF(b="Excellent","Green","")))))))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(dashboard): implement RC1 dashboard integration
</commit_message>
<xml_diff>
--- a/workbook/FinanceOS_v1.0.xlsx
+++ b/workbook/FinanceOS_v1.0.xlsx
@@ -89,6 +89,45 @@
     <definedName name="analysisLiquidityHealth">'Analysis Engine'!$B$163</definedName>
     <definedName name="analysisNetWorthHealth">'Analysis Engine'!$B$164</definedName>
     <definedName name="analysisCashFlowHealth">'Analysis Engine'!$B$165</definedName>
+    <definedName name="outNetWorth">'Business Engine'!$B$48</definedName>
+    <definedName name="outAssetValue">'Business Engine'!$B$35</definedName>
+    <definedName name="outOutstandingDebt">'Business Engine'!$B$42</definedName>
+    <definedName name="outTotalCash">'Business Engine'!$B$4</definedName>
+    <definedName name="outMonthlyIncome">'Business Engine'!$B$16</definedName>
+    <definedName name="outMonthlyExpense">'Business Engine'!$B$22</definedName>
+    <definedName name="outMonthlySavings">'Business Engine'!$B$29</definedName>
+    <definedName name="outSavingsRate">'Business Engine'!$B$30</definedName>
+    <definedName name="outMonthlyEMI">'Business Engine'!$B$43</definedName>
+    <definedName name="outGoalTarget">'Business Engine'!$B$53</definedName>
+    <definedName name="outGoalSaved">'Business Engine'!$B$54</definedName>
+    <definedName name="outGoalRemaining">'Business Engine'!$B$55</definedName>
+    <definedName name="outActiveGoalCount">'Business Engine'!$B$56</definedName>
+    <definedName name="outCompletedGoalCount">'Business Engine'!$B$57</definedName>
+    <definedName name="outGoalCompletion">'Business Engine'!$B$58</definedName>
+    <definedName name="outActiveLiabilityCount">'Business Engine'!$B$45</definedName>
+    <definedName name="outInvestmentValue">'Business Engine'!$B$70</definedName>
+    <definedName name="outPhysicalAssetValue">'Business Engine'!$B$71</definedName>
+    <definedName name="outPropertyValue">'Business Engine'!$B$72</definedName>
+    <definedName name="outRetirementAssetValue">'Business Engine'!$B$73</definedName>
+    <definedName name="outCashEquivalentValue">'Business Engine'!$B$74</definedName>
+    <definedName name="outOtherAssetValue">'Business Engine'!$B$75</definedName>
+    <definedName name="outActiveAssetCount">'Business Engine'!$B$38</definedName>
+    <definedName name="analysisSavingsHealthScore">'Analysis Engine'!$C$158</definedName>
+    <definedName name="analysisSavingsHealthSeverity">'Analysis Engine'!$D$158</definedName>
+    <definedName name="analysisExpenseHealthScore">'Analysis Engine'!$C$159</definedName>
+    <definedName name="analysisExpenseHealthSeverity">'Analysis Engine'!$D$159</definedName>
+    <definedName name="analysisDebtHealthScore">'Analysis Engine'!$C$160</definedName>
+    <definedName name="analysisDebtHealthSeverity">'Analysis Engine'!$D$160</definedName>
+    <definedName name="analysisAssetHealthScore">'Analysis Engine'!$C$161</definedName>
+    <definedName name="analysisAssetHealthSeverity">'Analysis Engine'!$D$161</definedName>
+    <definedName name="analysisGoalHealthScore">'Analysis Engine'!$C$162</definedName>
+    <definedName name="analysisGoalHealthSeverity">'Analysis Engine'!$D$162</definedName>
+    <definedName name="analysisLiquidityHealthScore">'Analysis Engine'!$C$163</definedName>
+    <definedName name="analysisLiquidityHealthSeverity">'Analysis Engine'!$D$163</definedName>
+    <definedName name="analysisNetWorthHealthScore">'Analysis Engine'!$C$164</definedName>
+    <definedName name="analysisNetWorthHealthSeverity">'Analysis Engine'!$D$164</definedName>
+    <definedName name="analysisCashFlowHealthScore">'Analysis Engine'!$C$165</definedName>
+    <definedName name="analysisCashFlowHealthSeverity">'Analysis Engine'!$D$165</definedName>
   </definedNames>
   <calcPr calcId="181029" forceFullCalc="1"/>
   <extLst>
@@ -100,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="405">
   <si>
     <t>Setting ID</t>
   </si>
@@ -1237,17 +1276,97 @@
   </si>
   <si>
     <t>Cash Flow Health</t>
+  </si>
+  <si>
+    <t>Financial Snapshot</t>
+  </si>
+  <si>
+    <t>Total Assets</t>
+  </si>
+  <si>
+    <t>Total Liabilities</t>
+  </si>
+  <si>
+    <t>Available Cash</t>
+  </si>
+  <si>
+    <t>Financial Health</t>
+  </si>
+  <si>
+    <t>Goal Progress</t>
+  </si>
+  <si>
+    <t>Total Target</t>
+  </si>
+  <si>
+    <t>Total Saved</t>
+  </si>
+  <si>
+    <t>Active Goals</t>
+  </si>
+  <si>
+    <t>Completed Goals</t>
+  </si>
+  <si>
+    <t>Completion</t>
+  </si>
+  <si>
+    <t>Physical Asset</t>
+  </si>
+  <si>
+    <t>Property</t>
+  </si>
+  <si>
+    <t>Retirement Asset</t>
+  </si>
+  <si>
+    <t>Cash Equivalent</t>
+  </si>
+  <si>
+    <t>Other Asset</t>
+  </si>
+  <si>
+    <t>Total Asset Value</t>
+  </si>
+  <si>
+    <t>Liability Summary</t>
+  </si>
+  <si>
+    <t>Outstanding Debt</t>
+  </si>
+  <si>
+    <t>Monthly EMI</t>
+  </si>
+  <si>
+    <t>Active Liabilities</t>
+  </si>
+  <si>
+    <t>Cash Flow Summary</t>
+  </si>
+  <si>
+    <t>Surplus</t>
+  </si>
+  <si>
+    <t>Monthly Overview</t>
+  </si>
+  <si>
+    <t>Reserved</t>
+  </si>
+  <si>
+    <t>Quick Insights</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="167" formatCode="dd/mm/yyyy hh:mm"/>
+    <numFmt numFmtId="168" formatCode="₹ #,##0.00"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -1295,7 +1414,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
@@ -1328,6 +1447,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12952,19 +13080,534 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="1" max="12" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>177</v>
       </c>
     </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>380</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" s="12">
+        <f>outNetWorth</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="12">
+        <f>outAssetValue</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="12">
+        <f>outOutstandingDebt</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="12">
+        <f>outTotalCash</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" s="12">
+        <f>outMonthlyIncome</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="12">
+        <f>outMonthlyExpense</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="12">
+        <f>outMonthlySavings</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="13">
+        <f>outSavingsRate</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15" s="0" t="str">
+        <f>analysisSavingsHealth</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="D15" s="0" t="str">
+        <f>analysisExpenseHealth</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="G15" s="0" t="str">
+        <f>analysisDebtHealth</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="J15" s="0" t="str">
+        <f>analysisAssetHealth</f>
+        <v>Unavailable</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" s="14" t="str">
+        <f>analysisSavingsHealthScore</f>
+        <v/>
+      </c>
+      <c r="D16" s="14" t="str">
+        <f>analysisExpenseHealthScore</f>
+        <v/>
+      </c>
+      <c r="G16" s="14" t="str">
+        <f>analysisDebtHealthScore</f>
+        <v/>
+      </c>
+      <c r="J16" s="14" t="str">
+        <f>analysisAssetHealthScore</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17" s="0" t="str">
+        <f>analysisSavingsHealthSeverity</f>
+        <v/>
+      </c>
+      <c r="D17" s="0" t="str">
+        <f>analysisExpenseHealthSeverity</f>
+        <v/>
+      </c>
+      <c r="G17" s="0" t="str">
+        <f>analysisDebtHealthSeverity</f>
+        <v/>
+      </c>
+      <c r="J17" s="0" t="str">
+        <f>analysisAssetHealthSeverity</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
+        <v>375</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>376</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" s="0" t="str">
+        <f>analysisGoalHealth</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="D20" s="0" t="str">
+        <f>analysisLiquidityHealth</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="G20" s="0" t="str">
+        <f>analysisNetWorthHealth</f>
+        <v>Unavailable</v>
+      </c>
+      <c r="J20" s="0" t="str">
+        <f>analysisCashFlowHealth</f>
+        <v>Unavailable</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21" s="14" t="str">
+        <f>analysisGoalHealthScore</f>
+        <v/>
+      </c>
+      <c r="D21" s="14" t="str">
+        <f>analysisLiquidityHealthScore</f>
+        <v/>
+      </c>
+      <c r="G21" s="14" t="str">
+        <f>analysisNetWorthHealthScore</f>
+        <v/>
+      </c>
+      <c r="J21" s="14" t="str">
+        <f>analysisCashFlowHealthScore</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22" s="0" t="str">
+        <f>analysisGoalHealthSeverity</f>
+        <v/>
+      </c>
+      <c r="D22" s="0" t="str">
+        <f>analysisLiquidityHealthSeverity</f>
+        <v/>
+      </c>
+      <c r="G22" s="0" t="str">
+        <f>analysisNetWorthHealthSeverity</f>
+        <v/>
+      </c>
+      <c r="J22" s="0" t="str">
+        <f>analysisCashFlowHealthSeverity</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>386</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A29" s="12">
+        <f>outGoalTarget</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="12">
+        <f>outGoalSaved</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="12">
+        <f>outGoalRemaining</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>387</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>388</v>
+      </c>
+      <c r="I31" s="9" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" s="14">
+        <f>outActiveGoalCount</f>
+        <v>0</v>
+      </c>
+      <c r="E32" s="14">
+        <f>outCompletedGoalCount</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="13">
+        <f>outGoalCompletion</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A37" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>390</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>392</v>
+      </c>
+      <c r="I37" s="9" t="s">
+        <v>393</v>
+      </c>
+      <c r="K37" s="9" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A38" s="12">
+        <f>outInvestmentValue</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="12">
+        <f>outPhysicalAssetValue</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="12">
+        <f>outPropertyValue</f>
+        <v>0</v>
+      </c>
+      <c r="G38" s="12">
+        <f>outRetirementAssetValue</f>
+        <v>0</v>
+      </c>
+      <c r="I38" s="12">
+        <f>outCashEquivalentValue</f>
+        <v>0</v>
+      </c>
+      <c r="K38" s="12">
+        <f>outOtherAssetValue</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A40" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="E40" s="12">
+        <f>outAssetValue</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="9" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="I41" s="14">
+        <f>outActiveAssetCount</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A45" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="I45" s="9" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A46" s="12">
+        <f>outOutstandingDebt</f>
+        <v>0</v>
+      </c>
+      <c r="E46" s="12">
+        <f>outMonthlyEMI</f>
+        <v>0</v>
+      </c>
+      <c r="I46" s="14">
+        <f>outActiveLiabilityCount</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A50" s="3" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A52" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="I52" s="9" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A53" s="12">
+        <f>outMonthlyIncome</f>
+        <v>0</v>
+      </c>
+      <c r="E53" s="12">
+        <f>outMonthlyExpense</f>
+        <v>0</v>
+      </c>
+      <c r="I53" s="12">
+        <f>outMonthlySavings</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A57" s="3" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A58" s="9" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A61" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A62" s="9" t="s">
+        <v>403</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <mergeCells count="99">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="A12:L12"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="E28:H28"/>
+    <mergeCell ref="I28:L28"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="E29:H29"/>
+    <mergeCell ref="I29:L29"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:L31"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="E32:H32"/>
+    <mergeCell ref="I32:L32"/>
+    <mergeCell ref="A35:L35"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="K38:L38"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="E40:H40"/>
+    <mergeCell ref="I40:L40"/>
+    <mergeCell ref="I41:L41"/>
+    <mergeCell ref="A43:L43"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="E45:H45"/>
+    <mergeCell ref="I45:L45"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="E46:H46"/>
+    <mergeCell ref="I46:L46"/>
+    <mergeCell ref="A50:L50"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="E52:H52"/>
+    <mergeCell ref="I52:L52"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="E53:H53"/>
+    <mergeCell ref="I53:L53"/>
+    <mergeCell ref="A57:L57"/>
+    <mergeCell ref="A58:L58"/>
+    <mergeCell ref="A61:L61"/>
+    <mergeCell ref="A62:L62"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(insights-engine): implement RC1 insights engine
</commit_message>
<xml_diff>
--- a/workbook/FinanceOS_v1.0.xlsx
+++ b/workbook/FinanceOS_v1.0.xlsx
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="419">
   <si>
     <t>Setting ID</t>
   </si>
@@ -1354,6 +1354,42 @@
   </si>
   <si>
     <t>Quick Insights</t>
+  </si>
+  <si>
+    <t>Headline</t>
+  </si>
+  <si>
+    <t>Explanation</t>
+  </si>
+  <si>
+    <t>Supporting Metric</t>
+  </si>
+  <si>
+    <t>Recommended Interpretation</t>
+  </si>
+  <si>
+    <t>INS-SAV</t>
+  </si>
+  <si>
+    <t>INS-EXP</t>
+  </si>
+  <si>
+    <t>INS-DEBT</t>
+  </si>
+  <si>
+    <t>INS-ASSET</t>
+  </si>
+  <si>
+    <t>INS-GOAL</t>
+  </si>
+  <si>
+    <t>INS-LIQ</t>
+  </si>
+  <si>
+    <t>INS-NW</t>
+  </si>
+  <si>
+    <t>INS-CF</t>
   </si>
 </sst>
 </file>
@@ -13615,19 +13651,605 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>178</v>
       </c>
     </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="str">
+        <f>IF(AND(analysisSavingsHealth="Unavailable",analysisExpenseHealth="Unavailable",analysisDebtHealth="Unavailable",analysisAssetHealth="Unavailable",analysisGoalHealth="Unavailable",analysisLiquidityHealth="Unavailable",analysisNetWorthHealth="Unavailable",analysisCashFlowHealth="Unavailable"),"No financial insights available yet.","")</f>
+        <v>No financial insights available yet.</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>370</v>
+      </c>
+      <c r="E7" t="str">
+        <f>LET(b,analysisSavingsHealth,IF(b="Unavailable","",analysisSavingsHealthSeverity))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" t="str">
+        <f>LET(b,analysisSavingsHealth,IF(b="Unavailable","","Savings"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E9" t="str">
+        <f>LET(b,analysisSavingsHealth,IF(b="Unavailable","",IF(b="Critical","Monthly savings are negative.",IF(b="Weak","Savings rate is Weak.",IF(b="Moderate","Savings rate is Moderate.",IF(b="Strong","Savings rate is Strong.",IF(b="Excellent","Savings rate is Excellent.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>406</v>
+      </c>
+      <c r="E10" t="str">
+        <f>LET(b,analysisSavingsHealth,IF(b="Unavailable","",IF(b="Critical","Income did not cover current-month expenses.",IF(b="Weak","Official savings rate is in the Weak band.",IF(b="Moderate","Official savings rate is in the Moderate band.",IF(b="Strong","Official savings rate is in the Strong band.",IF(b="Excellent","Official savings rate is in the Excellent band.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>407</v>
+      </c>
+      <c r="E11" t="str">
+        <f>LET(b,analysisSavingsHealth,IF(b="Unavailable","",IFERROR(TEXT(outSavingsRate,"0.0%"),"")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>408</v>
+      </c>
+      <c r="E12" t="str">
+        <f>LET(b,analysisSavingsHealth,IF(b="Unavailable","",IF(b="Critical","This month produced a cash deficit.",IF(b="Weak","Most income was absorbed by current-month expenses.",IF(b="Moderate","A surplus exists, but it is modest relative to income.",IF(b="Strong","Current-month cash flow left a solid surplus.",IF(b="Excellent","Current-month cash flow left a large surplus.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>370</v>
+      </c>
+      <c r="E15" t="str">
+        <f>LET(b,analysisExpenseHealth,IF(b="Unavailable","",analysisExpenseHealthSeverity))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" t="str">
+        <f>LET(b,analysisExpenseHealth,IF(b="Unavailable","","Expense"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>405</v>
+      </c>
+      <c r="E17" t="str">
+        <f>LET(b,analysisExpenseHealth,IF(b="Unavailable","",IF(b="Critical","Expense Health is Critical.",IF(b="Weak","Expense Health is Weak.",IF(b="Moderate","Expense Health is Moderate.",IF(b="Strong","Expense Health is Strong.",IF(b="Excellent","Expense Health is Excellent.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>406</v>
+      </c>
+      <c r="E18" t="str">
+        <f>LET(b,analysisExpenseHealth,IF(b="Unavailable","",IF(b="Critical","Current-month expenses are at or above income, or expenses exist with no income.",IF(b="Weak","Current-month expenses are high relative to income.",IF(b="Moderate","Current-month expenses are in the Moderate band versus income.",IF(b="Strong","Current-month expenses are in the Strong band versus income.",IF(b="Excellent","Current-month expenses are in the Excellent band versus income.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>407</v>
+      </c>
+      <c r="E19" t="str">
+        <f>LET(b,analysisExpenseHealth,IF(b="Unavailable","",IFERROR(TEXT(outMonthlyExpense,"₹ #,##0.00"),"")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>408</v>
+      </c>
+      <c r="E20" t="str">
+        <f>LET(b,analysisExpenseHealth,IF(b="Unavailable","",IF(b="Critical","Spending pressure is in the Critical band.",IF(b="Weak","Spending absorbed most of this month’s income.",IF(b="Moderate","Spending is material relative to income.",IF(b="Strong","Spending left room for a surplus.",IF(b="Excellent","Spending is low relative to income.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>370</v>
+      </c>
+      <c r="E23" t="str">
+        <f>LET(b,analysisDebtHealth,IF(b="Unavailable","",analysisDebtHealthSeverity))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" t="str">
+        <f>LET(b,analysisDebtHealth,IF(b="Unavailable","","Debt"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>405</v>
+      </c>
+      <c r="E25" t="str">
+        <f>LET(b,analysisDebtHealth,IF(b="Unavailable","",IF(b="Critical","Debt Health is Critical.",IF(b="Weak","Debt Health is Weak.",IF(b="Moderate","Debt Health is Moderate.",IF(b="Strong","Debt Health is Strong.",IF(b="Excellent","Debt Health is Excellent.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>406</v>
+      </c>
+      <c r="E26" t="str">
+        <f>LET(b,analysisDebtHealth,IF(b="Unavailable","",IF(b="Critical","EMI burden is in the Critical band.",IF(b="Weak","EMI burden is in the Weak band.",IF(b="Moderate","EMI burden is in the Moderate band.",IF(b="Strong","EMI burden is in the Strong band.",IF(b="Excellent","EMI burden is in the Excellent band, or there are no active liabilities.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>407</v>
+      </c>
+      <c r="E27" t="str">
+        <f>LET(b,analysisDebtHealth,IF(b="Unavailable","",IFERROR(TEXT(outOutstandingDebt,"₹ #,##0.00")&amp;" · "&amp;TEXT(outMonthlyEMI,"₹ #,##0.00"),"")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>408</v>
+      </c>
+      <c r="E28" t="str">
+        <f>LET(b,analysisDebtHealth,IF(b="Unavailable","",IF(b="Critical","Active debt service is heavy versus current-month income.",IF(b="Weak","Active debt service is elevated versus current-month income.",IF(b="Moderate","Active debt service is noticeable versus current-month income.",IF(b="Strong","Active debt service is limited versus current-month income.",IF(b="Excellent","Debt service is not a current pressure.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>370</v>
+      </c>
+      <c r="E31" t="str">
+        <f>LET(b,analysisAssetHealth,IF(b="Unavailable","",analysisAssetHealthSeverity))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="E32" t="str">
+        <f>LET(b,analysisAssetHealth,IF(b="Unavailable","","Asset"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>405</v>
+      </c>
+      <c r="E33" t="str">
+        <f>LET(b,analysisAssetHealth,IF(b="Unavailable","",IF(b="Critical","Asset Health is Critical.",IF(b="Weak","Asset Health is Weak.",IF(b="Moderate","Asset Health is Moderate.",IF(b="Strong","Asset Health is Strong.",IF(b="Excellent","Asset Health is Excellent.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>406</v>
+      </c>
+      <c r="E34" t="str">
+        <f>LET(b,analysisAssetHealth,IF(b="Unavailable","",IF(b="Critical","Active non-cash assets are concentrated.",IF(b="Weak","Active non-cash assets show limited diversification.",IF(b="Moderate","Active non-cash assets are somewhat diversified.",IF(b="Strong","Active non-cash assets are well diversified.",IF(b="Excellent","Active non-cash assets are broadly diversified.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>407</v>
+      </c>
+      <c r="E35" t="str">
+        <f>LET(b,analysisAssetHealth,IF(b="Unavailable","",IFERROR(TEXT(outAssetValue,"₹ #,##0.00")&amp;" · "&amp;TEXT(outActiveAssetCount,"0"),"")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>408</v>
+      </c>
+      <c r="E36" t="str">
+        <f>LET(b,analysisAssetHealth,IF(b="Unavailable","",IF(b="Critical","Diversification is in the Critical band.",IF(b="Weak","Diversification is in the Weak band.",IF(b="Moderate","Diversification is in the Moderate band.",IF(b="Strong","Diversification is in the Strong band.",IF(b="Excellent","Diversification is in the Excellent band.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>370</v>
+      </c>
+      <c r="E39" t="str">
+        <f>LET(b,analysisGoalHealth,IF(b="Unavailable","",analysisGoalHealthSeverity))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>63</v>
+      </c>
+      <c r="E40" t="str">
+        <f>LET(b,analysisGoalHealth,IF(b="Unavailable","","Goal"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>405</v>
+      </c>
+      <c r="E41" t="str">
+        <f>LET(b,analysisGoalHealth,IF(b="Unavailable","",IF(b="Critical","Goal Health is Critical.",IF(b="Weak","Goal Health is Weak.",IF(b="Moderate","Goal Health is Moderate.",IF(b="Strong","Goal Health is Strong.",IF(b="Excellent","Goal Health is Excellent.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>406</v>
+      </c>
+      <c r="E42" t="str">
+        <f>LET(b,analysisGoalHealth,IF(b="Unavailable","",IF(b="Critical","Active and completed goals have no recorded progress.",IF(b="Weak","Aggregate goal completion is in the Weak band.",IF(b="Moderate","Aggregate goal completion is in the Moderate band.",IF(b="Strong","Aggregate goal completion is in the Strong band.",IF(b="Excellent","Aggregate goal completion is in the Excellent band.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>407</v>
+      </c>
+      <c r="E43" t="str">
+        <f>LET(b,analysisGoalHealth,IF(b="Unavailable","",IFERROR(TEXT(outGoalCompletion,"0.0%"),"")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>408</v>
+      </c>
+      <c r="E44" t="str">
+        <f>LET(b,analysisGoalHealth,IF(b="Unavailable","",IF(b="Critical","Aggregate goal completion is in the Critical band.",IF(b="Weak","Some progress exists, but it is small versus targets.",IF(b="Moderate","Goal funding is underway.",IF(b="Strong","Goals are largely funded.",IF(b="Excellent","Goals are near or at target in aggregate.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>370</v>
+      </c>
+      <c r="E47" t="str">
+        <f>LET(b,analysisLiquidityHealth,IF(b="Unavailable","",analysisLiquidityHealthSeverity))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>63</v>
+      </c>
+      <c r="E48" t="str">
+        <f>LET(b,analysisLiquidityHealth,IF(b="Unavailable","","Liquidity"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>405</v>
+      </c>
+      <c r="E49" t="str">
+        <f>LET(b,analysisLiquidityHealth,IF(b="Unavailable","",IF(b="Critical","Liquidity Health is Critical.",IF(b="Weak","Liquidity Health is Weak.",IF(b="Moderate","Liquidity Health is Moderate.",IF(b="Strong","",IF(b="Healthy","Liquidity Health is Healthy.",IF(b="Excellent","Liquidity Health is Excellent.",""))))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>406</v>
+      </c>
+      <c r="E50" t="str">
+        <f>LET(b,analysisLiquidityHealth,IF(b="Unavailable","",IF(b="Critical","Available cash is low relative to current-month expenses.",IF(b="Weak","Available cash is limited relative to current-month expenses.",IF(b="Moderate","Available cash is moderate relative to current-month expenses.",IF(b="Strong","",IF(b="Healthy","Available cash is in the Healthy band relative to current-month expenses.",IF(b="Excellent","Available cash is strong relative to current-month expenses, or expenses are zero with cash on hand.",""))))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>407</v>
+      </c>
+      <c r="E51" t="str">
+        <f>LET(b,analysisLiquidityHealth,IF(b="Unavailable","",IFERROR(TEXT(outTotalCash,"₹ #,##0.00")&amp;" · "&amp;TEXT(outMonthlyExpense,"₹ #,##0.00"),"")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>408</v>
+      </c>
+      <c r="E52" t="str">
+        <f>LET(b,analysisLiquidityHealth,IF(b="Unavailable","",IF(b="Critical","Cash coverage is in the Critical band.",IF(b="Weak","Cash coverage is in the Weak band.",IF(b="Moderate","Cash coverage is in the Moderate band.",IF(b="Strong","",IF(b="Healthy","Cash coverage is in the Healthy band.",IF(b="Excellent","Cash coverage is in the Excellent band.",""))))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>370</v>
+      </c>
+      <c r="E55" t="str">
+        <f>LET(b,analysisNetWorthHealth,IF(b="Unavailable","",analysisNetWorthHealthSeverity))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>63</v>
+      </c>
+      <c r="E56" t="str">
+        <f>LET(b,analysisNetWorthHealth,IF(b="Unavailable","","Net Worth"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>405</v>
+      </c>
+      <c r="E57" t="str">
+        <f>LET(b,analysisNetWorthHealth,IF(b="Unavailable","",IF(b="Critical","Net Worth Health is Critical.",IF(b="Weak","Net Worth Health is Weak.",IF(b="Moderate","Net Worth Health is Moderate.",IF(b="Strong","Net Worth Health is Strong.",IF(b="Excellent","Net Worth Health is Excellent.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>406</v>
+      </c>
+      <c r="E58" t="str">
+        <f>LET(b,analysisNetWorthHealth,IF(b="Unavailable","",IF(b="Critical","Official net worth is negative.",IF(b="Weak","Official net worth is in the Weak band.",IF(b="Moderate","Official net worth is in the Moderate band.",IF(b="Strong","Official net worth is in the Strong band.",IF(b="Excellent","Official net worth is in the Excellent band.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>407</v>
+      </c>
+      <c r="E59" t="str">
+        <f>LET(b,analysisNetWorthHealth,IF(b="Unavailable","",IFERROR(TEXT(outNetWorth,"₹ #,##0.00"),"")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>408</v>
+      </c>
+      <c r="E60" t="str">
+        <f>LET(b,analysisNetWorthHealth,IF(b="Unavailable","",IF(b="Critical","Liabilities exceed cash and active assets.",IF(b="Weak","Net worth is zero or leveraged.",IF(b="Moderate","Net worth is positive with moderate leverage.",IF(b="Strong","Net worth is positive with low leverage.",IF(b="Excellent","Net worth is positive with very low leverage.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>370</v>
+      </c>
+      <c r="E63" t="str">
+        <f>LET(b,analysisCashFlowHealth,IF(b="Unavailable","",analysisCashFlowHealthSeverity))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>63</v>
+      </c>
+      <c r="E64" t="str">
+        <f>LET(b,analysisCashFlowHealth,IF(b="Unavailable","","Cash Flow"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>405</v>
+      </c>
+      <c r="E65" t="str">
+        <f>LET(b,analysisCashFlowHealth,IF(b="Unavailable","",IF(b="Critical","Cash Flow Health is Critical.",IF(b="Weak","Cash Flow Health is Weak.",IF(b="Moderate","Cash Flow Health is Moderate.",IF(b="Strong","Cash Flow Health is Strong.",IF(b="Excellent","Cash Flow Health is Excellent.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>406</v>
+      </c>
+      <c r="E66" t="str">
+        <f>LET(b,analysisCashFlowHealth,IF(b="Unavailable","",IF(b="Critical","Current-month surplus is negative.",IF(b="Weak","Current-month surplus is zero.",IF(b="Moderate","Current-month surplus is in the Moderate band.",IF(b="Strong","Current-month surplus is in the Strong band.",IF(b="Excellent","Current-month surplus is in the Excellent band.","")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>407</v>
+      </c>
+      <c r="E67" t="str">
+        <f>LET(b,analysisCashFlowHealth,IF(b="Unavailable","",IFERROR(TEXT(outMonthlySavings,"₹ #,##0.00"),"")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>408</v>
+      </c>
+      <c r="E68" t="str">
+        <f>LET(b,analysisCashFlowHealth,IF(b="Unavailable","",IF(b="Critical","Cash flow produced a deficit.",IF(b="Weak","Income and expenses offset.",IF(b="Moderate","A small surplus exists.",IF(b="Strong","Cash flow produced a solid surplus.",IF(b="Excellent","Cash flow produced a large surplus.","")))))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <mergeCells count="106">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="E7:L7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="E8:L8"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="E9:L9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="E10:L10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:L11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="E12:L12"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="E15:L15"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="E16:L16"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="E17:L17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="E18:L18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="E19:L19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="E20:L20"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="E23:L23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="E24:L24"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="E25:L25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="E26:L26"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="E27:L27"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="E28:L28"/>
+    <mergeCell ref="A30:L30"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="E31:L31"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="E32:L32"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="E33:L33"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="E34:L34"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="E35:L35"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="E36:L36"/>
+    <mergeCell ref="A38:L38"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="E39:L39"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="E40:L40"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="E41:L41"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="E42:L42"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="E43:L43"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="E44:L44"/>
+    <mergeCell ref="A46:L46"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="E47:L47"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="E48:L48"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="E49:L49"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="E50:L50"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="E51:L51"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="E52:L52"/>
+    <mergeCell ref="A54:L54"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="E55:L55"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="E56:L56"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="E57:L57"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="E58:L58"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="E59:L59"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="E60:L60"/>
+    <mergeCell ref="A62:L62"/>
+    <mergeCell ref="A63:D63"/>
+    <mergeCell ref="E63:L63"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="E64:L64"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="E65:L65"/>
+    <mergeCell ref="A66:D66"/>
+    <mergeCell ref="E66:L66"/>
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="E67:L67"/>
+    <mergeCell ref="A68:D68"/>
+    <mergeCell ref="E68:L68"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>